<commit_message>
Update employment causality analysis
r2
</commit_message>
<xml_diff>
--- a/employment/03_substitution_analysis.xlsx
+++ b/employment/03_substitution_analysis.xlsx
@@ -604,7 +604,7 @@
       <c r="D2" s="6" t="inlineStr">
         <is>
           <t>Emp
-2016</t>
+2019</t>
         </is>
       </c>
       <c r="E2" s="6" t="inlineStr">
@@ -626,7 +626,7 @@
       <c r="H2" s="7" t="inlineStr">
         <is>
           <t>Emp
-2016</t>
+2019</t>
         </is>
       </c>
       <c r="I2" s="7" t="inlineStr">
@@ -648,7 +648,7 @@
       <c r="L2" s="8" t="inlineStr">
         <is>
           <t>Emp
-2016</t>
+2019</t>
         </is>
       </c>
       <c r="M2" s="8" t="inlineStr">
@@ -695,40 +695,40 @@
         <v>8.942662</v>
       </c>
       <c r="D3" s="12" t="n">
-        <v>33241.5</v>
+        <v>36459.75</v>
       </c>
       <c r="E3" s="12" t="n">
         <v>47316</v>
       </c>
       <c r="F3" s="13" t="n">
-        <v>14074.5</v>
+        <v>10856.25</v>
       </c>
       <c r="G3" s="14" t="n">
-        <v>0.4234014710527503</v>
+        <v>0.2977598584740707</v>
       </c>
       <c r="H3" s="12" t="n">
-        <v>204296.75</v>
+        <v>207845.5</v>
       </c>
       <c r="I3" s="12" t="n">
         <v>227371.75</v>
       </c>
       <c r="J3" s="13" t="n">
-        <v>23075</v>
+        <v>19526.25</v>
       </c>
       <c r="K3" s="14" t="n">
-        <v>0.1129484438690287</v>
+        <v>0.09394598391593756</v>
       </c>
       <c r="L3" s="12" t="n">
-        <v>81601.25</v>
+        <v>76834.5</v>
       </c>
       <c r="M3" s="12" t="n">
         <v>78831.25</v>
       </c>
       <c r="N3" s="13" t="n">
-        <v>-2770</v>
+        <v>1996.75</v>
       </c>
       <c r="O3" s="14" t="n">
-        <v>-0.03394555843200931</v>
+        <v>0.02598767480754088</v>
       </c>
       <c r="P3" s="10" t="inlineStr">
         <is>
@@ -737,7 +737,7 @@
       </c>
       <c r="Q3" s="10" t="inlineStr">
         <is>
-          <t>Decline</t>
+          <t>Stable/Growth</t>
         </is>
       </c>
     </row>
@@ -756,40 +756,40 @@
         <v>8.239623999999999</v>
       </c>
       <c r="D4" s="12" t="n">
-        <v>11038.75</v>
+        <v>13353.25</v>
       </c>
       <c r="E4" s="12" t="n">
         <v>19382.75</v>
       </c>
       <c r="F4" s="13" t="n">
-        <v>8344</v>
+        <v>6029.5</v>
       </c>
       <c r="G4" s="14" t="n">
-        <v>0.7558826859925263</v>
+        <v>0.4515380150899594</v>
       </c>
       <c r="H4" s="12" t="n">
-        <v>69401.25</v>
+        <v>68727.25</v>
       </c>
       <c r="I4" s="12" t="n">
         <v>71449.25</v>
       </c>
       <c r="J4" s="13" t="n">
-        <v>2048</v>
+        <v>2722</v>
       </c>
       <c r="K4" s="14" t="n">
-        <v>0.02950955494317465</v>
+        <v>0.03960583320298717</v>
       </c>
       <c r="L4" s="12" t="n">
-        <v>25559</v>
+        <v>22017.75</v>
       </c>
       <c r="M4" s="12" t="n">
         <v>18775.5</v>
       </c>
       <c r="N4" s="13" t="n">
-        <v>-6783.5</v>
+        <v>-3242.25</v>
       </c>
       <c r="O4" s="14" t="n">
-        <v>-0.2654055322978207</v>
+        <v>-0.1472561910276936</v>
       </c>
       <c r="P4" s="10" t="inlineStr">
         <is>
@@ -817,40 +817,40 @@
         <v>4.588372000000001</v>
       </c>
       <c r="D5" s="12" t="n">
-        <v>3948.75</v>
+        <v>5658.25</v>
       </c>
       <c r="E5" s="12" t="n">
         <v>8055</v>
       </c>
       <c r="F5" s="13" t="n">
-        <v>4106.25</v>
+        <v>2396.75</v>
       </c>
       <c r="G5" s="14" t="n">
-        <v>1.03988603988604</v>
+        <v>0.4235850307073742</v>
       </c>
       <c r="H5" s="12" t="n">
-        <v>34785.5</v>
+        <v>36636.25</v>
       </c>
       <c r="I5" s="12" t="n">
         <v>37579.5</v>
       </c>
       <c r="J5" s="13" t="n">
-        <v>2794</v>
+        <v>943.25</v>
       </c>
       <c r="K5" s="14" t="n">
-        <v>0.08032082333156057</v>
+        <v>0.02574635777406258</v>
       </c>
       <c r="L5" s="12" t="n">
-        <v>5546.25</v>
+        <v>5179.25</v>
       </c>
       <c r="M5" s="12" t="n">
         <v>3963.75</v>
       </c>
       <c r="N5" s="13" t="n">
-        <v>-1582.5</v>
+        <v>-1215.5</v>
       </c>
       <c r="O5" s="14" t="n">
-        <v>-0.2853279242731576</v>
+        <v>-0.2346864893565671</v>
       </c>
       <c r="P5" s="10" t="inlineStr">
         <is>
@@ -878,44 +878,44 @@
         <v>3.473613</v>
       </c>
       <c r="D6" s="12" t="n">
-        <v>38885.5</v>
+        <v>51296.75</v>
       </c>
       <c r="E6" s="12" t="n">
         <v>76245.75</v>
       </c>
       <c r="F6" s="13" t="n">
-        <v>37360.25</v>
+        <v>24949</v>
       </c>
       <c r="G6" s="14" t="n">
-        <v>0.9607758676113204</v>
+        <v>0.4863660953179295</v>
       </c>
       <c r="H6" s="12" t="n">
-        <v>671800.5</v>
+        <v>734265.75</v>
       </c>
       <c r="I6" s="12" t="n">
         <v>730032.5</v>
       </c>
       <c r="J6" s="13" t="n">
-        <v>58232</v>
+        <v>-4233.25</v>
       </c>
       <c r="K6" s="14" t="n">
-        <v>0.08668049517676751</v>
+        <v>-0.00576528320979155</v>
       </c>
       <c r="L6" s="12" t="n">
-        <v>76721</v>
+        <v>63919</v>
       </c>
       <c r="M6" s="12" t="n">
         <v>50936.5</v>
       </c>
       <c r="N6" s="13" t="n">
-        <v>-25784.5</v>
+        <v>-12982.5</v>
       </c>
       <c r="O6" s="14" t="n">
-        <v>-0.3360813858004979</v>
+        <v>-0.2031086218495283</v>
       </c>
       <c r="P6" s="10" t="inlineStr">
         <is>
-          <t>Net new jobs</t>
+          <t>Substitution</t>
         </is>
       </c>
       <c r="Q6" s="10" t="inlineStr">
@@ -939,40 +939,40 @@
         <v>2.805081</v>
       </c>
       <c r="D7" s="12" t="n">
-        <v>9607.25</v>
+        <v>10552.75</v>
       </c>
       <c r="E7" s="12" t="n">
         <v>15356</v>
       </c>
       <c r="F7" s="13" t="n">
-        <v>5748.75</v>
+        <v>4803.25</v>
       </c>
       <c r="G7" s="14" t="n">
-        <v>0.5983762262874391</v>
+        <v>0.4551657150979602</v>
       </c>
       <c r="H7" s="12" t="n">
-        <v>102705.5</v>
+        <v>97058.5</v>
       </c>
       <c r="I7" s="12" t="n">
         <v>89958.75</v>
       </c>
       <c r="J7" s="13" t="n">
-        <v>-12746.75</v>
+        <v>-7099.75</v>
       </c>
       <c r="K7" s="14" t="n">
-        <v>-0.1241097117486405</v>
+        <v>-0.07314918322455015</v>
       </c>
       <c r="L7" s="12" t="n">
-        <v>31955.25</v>
+        <v>25112.25</v>
       </c>
       <c r="M7" s="12" t="n">
         <v>18228.5</v>
       </c>
       <c r="N7" s="13" t="n">
-        <v>-13726.75</v>
+        <v>-6883.75</v>
       </c>
       <c r="O7" s="14" t="n">
-        <v>-0.4295616526235908</v>
+        <v>-0.2741192047705801</v>
       </c>
       <c r="P7" s="10" t="inlineStr">
         <is>
@@ -1000,40 +1000,40 @@
         <v>2.55925</v>
       </c>
       <c r="D8" s="12" t="n">
-        <v>9064.75</v>
+        <v>12587</v>
       </c>
       <c r="E8" s="12" t="n">
         <v>23823</v>
       </c>
       <c r="F8" s="13" t="n">
-        <v>14758.25</v>
+        <v>11236</v>
       </c>
       <c r="G8" s="14" t="n">
-        <v>1.628092335695965</v>
+        <v>0.8926670374195599</v>
       </c>
       <c r="H8" s="12" t="n">
-        <v>115357.5</v>
+        <v>121740.5</v>
       </c>
       <c r="I8" s="12" t="n">
         <v>128801.75</v>
       </c>
       <c r="J8" s="13" t="n">
-        <v>13444.25</v>
+        <v>7061.25</v>
       </c>
       <c r="K8" s="14" t="n">
-        <v>0.1165442212253213</v>
+        <v>0.05800247247218469</v>
       </c>
       <c r="L8" s="12" t="n">
-        <v>47632.5</v>
+        <v>40880</v>
       </c>
       <c r="M8" s="12" t="n">
         <v>34363</v>
       </c>
       <c r="N8" s="13" t="n">
-        <v>-13269.5</v>
+        <v>-6517</v>
       </c>
       <c r="O8" s="14" t="n">
-        <v>-0.278580800923739</v>
+        <v>-0.1594178082191781</v>
       </c>
       <c r="P8" s="10" t="inlineStr">
         <is>
@@ -1061,40 +1061,40 @@
         <v>2.434877</v>
       </c>
       <c r="D9" s="12" t="n">
-        <v>6641.5</v>
+        <v>8350</v>
       </c>
       <c r="E9" s="12" t="n">
         <v>11627</v>
       </c>
       <c r="F9" s="13" t="n">
-        <v>4985.5</v>
+        <v>3277</v>
       </c>
       <c r="G9" s="14" t="n">
-        <v>0.7506587367311601</v>
+        <v>0.3924550898203593</v>
       </c>
       <c r="H9" s="12" t="n">
-        <v>73169.75</v>
+        <v>72140.5</v>
       </c>
       <c r="I9" s="12" t="n">
         <v>67882</v>
       </c>
       <c r="J9" s="13" t="n">
-        <v>-5287.75</v>
+        <v>-4258.5</v>
       </c>
       <c r="K9" s="14" t="n">
-        <v>-0.07226688624739049</v>
+        <v>-0.05903064159522044</v>
       </c>
       <c r="L9" s="12" t="n">
-        <v>24497.5</v>
+        <v>24094</v>
       </c>
       <c r="M9" s="12" t="n">
         <v>20227</v>
       </c>
       <c r="N9" s="13" t="n">
-        <v>-4270.5</v>
+        <v>-3867</v>
       </c>
       <c r="O9" s="14" t="n">
-        <v>-0.1743239106031228</v>
+        <v>-0.1604963891425251</v>
       </c>
       <c r="P9" s="10" t="inlineStr">
         <is>
@@ -1122,44 +1122,44 @@
         <v>2.392509</v>
       </c>
       <c r="D10" s="12" t="n">
-        <v>8529.25</v>
+        <v>9851</v>
       </c>
       <c r="E10" s="12" t="n">
         <v>11946.5</v>
       </c>
       <c r="F10" s="13" t="n">
-        <v>3417.25</v>
+        <v>2095.5</v>
       </c>
       <c r="G10" s="14" t="n">
-        <v>0.4006507019960723</v>
+        <v>0.2127195208608263</v>
       </c>
       <c r="H10" s="12" t="n">
-        <v>45130.5</v>
+        <v>49423.5</v>
       </c>
       <c r="I10" s="12" t="n">
         <v>50194.75</v>
       </c>
       <c r="J10" s="13" t="n">
-        <v>5064.25</v>
+        <v>771.25</v>
       </c>
       <c r="K10" s="14" t="n">
-        <v>0.1122134698263924</v>
+        <v>0.01560492478274505</v>
       </c>
       <c r="L10" s="12" t="n">
-        <v>15105.5</v>
+        <v>16073.75</v>
       </c>
       <c r="M10" s="12" t="n">
         <v>11782.75</v>
       </c>
       <c r="N10" s="13" t="n">
-        <v>-3322.75</v>
+        <v>-4291</v>
       </c>
       <c r="O10" s="14" t="n">
-        <v>-0.2199695475158055</v>
+        <v>-0.2669569951007077</v>
       </c>
       <c r="P10" s="10" t="inlineStr">
         <is>
-          <t>Net new jobs</t>
+          <t>Substitution</t>
         </is>
       </c>
       <c r="Q10" s="10" t="inlineStr">
@@ -1183,44 +1183,44 @@
         <v>2.237543</v>
       </c>
       <c r="D11" s="12" t="n">
-        <v>3091.25</v>
+        <v>3459.25</v>
       </c>
       <c r="E11" s="12" t="n">
         <v>3348.5</v>
       </c>
       <c r="F11" s="13" t="n">
-        <v>257.25</v>
+        <v>-110.75</v>
       </c>
       <c r="G11" s="14" t="n">
-        <v>0.08321876263647392</v>
+        <v>-0.0320156103201561</v>
       </c>
       <c r="H11" s="12" t="n">
-        <v>22338.5</v>
+        <v>20899.5</v>
       </c>
       <c r="I11" s="12" t="n">
         <v>17900.5</v>
       </c>
       <c r="J11" s="13" t="n">
-        <v>-4438</v>
+        <v>-2999</v>
       </c>
       <c r="K11" s="14" t="n">
-        <v>-0.1986704568346129</v>
+        <v>-0.1434962558912893</v>
       </c>
       <c r="L11" s="12" t="n">
-        <v>6507.5</v>
+        <v>5687.75</v>
       </c>
       <c r="M11" s="12" t="n">
         <v>5047</v>
       </c>
       <c r="N11" s="13" t="n">
-        <v>-1460.5</v>
+        <v>-640.75</v>
       </c>
       <c r="O11" s="14" t="n">
-        <v>-0.2244333461390703</v>
+        <v>-0.1126543888180739</v>
       </c>
       <c r="P11" s="10" t="inlineStr">
         <is>
-          <t>Substitution</t>
+          <t>DC declining</t>
         </is>
       </c>
       <c r="Q11" s="10" t="inlineStr">
@@ -1244,40 +1244,40 @@
         <v>1.900304</v>
       </c>
       <c r="D12" s="12" t="n">
-        <v>9019</v>
+        <v>13382.25</v>
       </c>
       <c r="E12" s="12" t="n">
         <v>22821</v>
       </c>
       <c r="F12" s="13" t="n">
-        <v>13802</v>
+        <v>9438.75</v>
       </c>
       <c r="G12" s="14" t="n">
-        <v>1.530324869719481</v>
+        <v>0.705318612340974</v>
       </c>
       <c r="H12" s="12" t="n">
-        <v>127577.75</v>
+        <v>148345.25</v>
       </c>
       <c r="I12" s="12" t="n">
         <v>173738.5</v>
       </c>
       <c r="J12" s="13" t="n">
-        <v>46160.75</v>
+        <v>25393.25</v>
       </c>
       <c r="K12" s="14" t="n">
-        <v>0.3618244560669866</v>
+        <v>0.1711766976023836</v>
       </c>
       <c r="L12" s="12" t="n">
-        <v>21661</v>
+        <v>20125</v>
       </c>
       <c r="M12" s="12" t="n">
         <v>16161.75</v>
       </c>
       <c r="N12" s="13" t="n">
-        <v>-5499.25</v>
+        <v>-3963.25</v>
       </c>
       <c r="O12" s="14" t="n">
-        <v>-0.2538779373066802</v>
+        <v>-0.1969316770186335</v>
       </c>
       <c r="P12" s="10" t="inlineStr">
         <is>
@@ -1305,49 +1305,49 @@
         <v>1.594719</v>
       </c>
       <c r="D13" s="12" t="n">
-        <v>14147.75</v>
+        <v>10570.5</v>
       </c>
       <c r="E13" s="12" t="n">
         <v>11933.5</v>
       </c>
       <c r="F13" s="13" t="n">
-        <v>-2214.25</v>
+        <v>1363</v>
       </c>
       <c r="G13" s="14" t="n">
-        <v>-0.1565089855277341</v>
+        <v>0.1289437585733882</v>
       </c>
       <c r="H13" s="12" t="n">
-        <v>79755.25</v>
+        <v>74603.25</v>
       </c>
       <c r="I13" s="12" t="n">
         <v>82062</v>
       </c>
       <c r="J13" s="13" t="n">
-        <v>2306.75</v>
+        <v>7458.75</v>
       </c>
       <c r="K13" s="14" t="n">
-        <v>0.02892286087749709</v>
+        <v>0.09997888831920862</v>
       </c>
       <c r="L13" s="12" t="n">
-        <v>26572.25</v>
+        <v>23721.5</v>
       </c>
       <c r="M13" s="12" t="n">
         <v>21836.75</v>
       </c>
       <c r="N13" s="13" t="n">
-        <v>-4735.5</v>
+        <v>-1884.75</v>
       </c>
       <c r="O13" s="14" t="n">
-        <v>-0.1782122326863551</v>
+        <v>-0.07945323862318994</v>
       </c>
       <c r="P13" s="10" t="inlineStr">
         <is>
-          <t>DC declining</t>
+          <t>Net new jobs</t>
         </is>
       </c>
       <c r="Q13" s="10" t="inlineStr">
         <is>
-          <t>Large decline</t>
+          <t>Decline</t>
         </is>
       </c>
     </row>
@@ -1366,44 +1366,44 @@
         <v>1.512326</v>
       </c>
       <c r="D14" s="12" t="n">
-        <v>8716.75</v>
+        <v>9784.5</v>
       </c>
       <c r="E14" s="12" t="n">
         <v>13362.75</v>
       </c>
       <c r="F14" s="13" t="n">
-        <v>4646</v>
+        <v>3578.25</v>
       </c>
       <c r="G14" s="14" t="n">
-        <v>0.5329968164740299</v>
+        <v>0.3657059635137207</v>
       </c>
       <c r="H14" s="12" t="n">
-        <v>88182.75</v>
+        <v>90644.25</v>
       </c>
       <c r="I14" s="12" t="n">
         <v>93065</v>
       </c>
       <c r="J14" s="13" t="n">
-        <v>4882.25</v>
+        <v>2420.75</v>
       </c>
       <c r="K14" s="14" t="n">
-        <v>0.05536513660551525</v>
+        <v>0.02670605140425344</v>
       </c>
       <c r="L14" s="12" t="n">
-        <v>29335.5</v>
+        <v>28645</v>
       </c>
       <c r="M14" s="12" t="n">
         <v>26767.25</v>
       </c>
       <c r="N14" s="13" t="n">
-        <v>-2568.25</v>
+        <v>-1877.75</v>
       </c>
       <c r="O14" s="14" t="n">
-        <v>-0.08754751069523274</v>
+        <v>-0.06555245243497992</v>
       </c>
       <c r="P14" s="10" t="inlineStr">
         <is>
-          <t>Net new jobs</t>
+          <t>Substitution</t>
         </is>
       </c>
       <c r="Q14" s="10" t="inlineStr">
@@ -1427,40 +1427,40 @@
         <v>1.468625</v>
       </c>
       <c r="D15" s="12" t="n">
-        <v>518</v>
+        <v>487.25</v>
       </c>
       <c r="E15" s="12" t="n">
         <v>313.5</v>
       </c>
       <c r="F15" s="13" t="n">
-        <v>-204.5</v>
+        <v>-173.75</v>
       </c>
       <c r="G15" s="14" t="n">
-        <v>-0.3947876447876448</v>
+        <v>-0.3565931246793227</v>
       </c>
       <c r="H15" s="12" t="n">
-        <v>6896.75</v>
+        <v>6253.75</v>
       </c>
       <c r="I15" s="12" t="n">
         <v>5539</v>
       </c>
       <c r="J15" s="13" t="n">
-        <v>-1357.75</v>
+        <v>-714.75</v>
       </c>
       <c r="K15" s="14" t="n">
-        <v>-0.1968680900424113</v>
+        <v>-0.1142914251449131</v>
       </c>
       <c r="L15" s="12" t="n">
-        <v>1871.5</v>
+        <v>1777.75</v>
       </c>
       <c r="M15" s="12" t="n">
         <v>1985.5</v>
       </c>
       <c r="N15" s="13" t="n">
-        <v>114</v>
+        <v>207.75</v>
       </c>
       <c r="O15" s="14" t="n">
-        <v>0.06091370558375635</v>
+        <v>0.1168612009562649</v>
       </c>
       <c r="P15" s="10" t="inlineStr">
         <is>
@@ -1488,40 +1488,40 @@
         <v>1.449626</v>
       </c>
       <c r="D16" s="12" t="n">
-        <v>1669</v>
+        <v>2342.5</v>
       </c>
       <c r="E16" s="12" t="n">
         <v>2935.25</v>
       </c>
       <c r="F16" s="13" t="n">
-        <v>1266.25</v>
+        <v>592.75</v>
       </c>
       <c r="G16" s="14" t="n">
-        <v>0.7586878370281606</v>
+        <v>0.2530416221985058</v>
       </c>
       <c r="H16" s="12" t="n">
-        <v>14868.5</v>
+        <v>16906.75</v>
       </c>
       <c r="I16" s="12" t="n">
         <v>21858.75</v>
       </c>
       <c r="J16" s="13" t="n">
-        <v>6990.25</v>
+        <v>4952</v>
       </c>
       <c r="K16" s="14" t="n">
-        <v>0.4701382116555133</v>
+        <v>0.2929007644875568</v>
       </c>
       <c r="L16" s="12" t="n">
-        <v>3973.25</v>
+        <v>4065</v>
       </c>
       <c r="M16" s="12" t="n">
         <v>3633.25</v>
       </c>
       <c r="N16" s="13" t="n">
-        <v>-340</v>
+        <v>-431.75</v>
       </c>
       <c r="O16" s="14" t="n">
-        <v>-0.08557226451897061</v>
+        <v>-0.1062115621156212</v>
       </c>
       <c r="P16" s="10" t="inlineStr">
         <is>
@@ -1530,7 +1530,7 @@
       </c>
       <c r="Q16" s="10" t="inlineStr">
         <is>
-          <t>Decline</t>
+          <t>Large decline</t>
         </is>
       </c>
     </row>
@@ -1549,40 +1549,40 @@
         <v>1.256079</v>
       </c>
       <c r="D17" s="12" t="n">
-        <v>4642.25</v>
+        <v>4020.5</v>
       </c>
       <c r="E17" s="12" t="n">
         <v>1887.75</v>
       </c>
       <c r="F17" s="13" t="n">
-        <v>-2754.5</v>
+        <v>-2132.75</v>
       </c>
       <c r="G17" s="14" t="n">
-        <v>-0.5933545155905003</v>
+        <v>-0.5304688471583137</v>
       </c>
       <c r="H17" s="12" t="n">
-        <v>18448.75</v>
+        <v>17148.75</v>
       </c>
       <c r="I17" s="12" t="n">
         <v>18053</v>
       </c>
       <c r="J17" s="13" t="n">
-        <v>-395.75</v>
+        <v>904.25</v>
       </c>
       <c r="K17" s="14" t="n">
-        <v>-0.02145131783996206</v>
+        <v>0.0527297908010788</v>
       </c>
       <c r="L17" s="12" t="n">
-        <v>3551.25</v>
+        <v>3318.75</v>
       </c>
       <c r="M17" s="12" t="n">
         <v>3071.25</v>
       </c>
       <c r="N17" s="13" t="n">
-        <v>-480</v>
+        <v>-247.5</v>
       </c>
       <c r="O17" s="14" t="n">
-        <v>-0.1351636747624076</v>
+        <v>-0.07457627118644068</v>
       </c>
       <c r="P17" s="10" t="inlineStr">
         <is>
@@ -1591,7 +1591,7 @@
       </c>
       <c r="Q17" s="10" t="inlineStr">
         <is>
-          <t>Large decline</t>
+          <t>Decline</t>
         </is>
       </c>
     </row>
@@ -1607,43 +1607,43 @@
         </is>
       </c>
       <c r="C18" s="11" t="n">
-        <v>56.613435</v>
+        <v>56.595705</v>
       </c>
       <c r="D18" s="12" t="n">
-        <v>300874.25</v>
+        <v>333652.25</v>
       </c>
       <c r="E18" s="12" t="n">
-        <v>464954.8333333333</v>
+        <v>464389.0833333333</v>
       </c>
       <c r="F18" s="13" t="n">
-        <v>164080.5833333333</v>
+        <v>130736.8333333333</v>
       </c>
       <c r="G18" s="14" t="n">
-        <v>0.5453460485014364</v>
+        <v>0.3918356112789089</v>
       </c>
       <c r="H18" s="12" t="n">
-        <v>3026759.5</v>
+        <v>3062567</v>
       </c>
       <c r="I18" s="12" t="n">
-        <v>3114983.25</v>
+        <v>3104060.75</v>
       </c>
       <c r="J18" s="13" t="n">
-        <v>88223.75</v>
+        <v>41493.75</v>
       </c>
       <c r="K18" s="14" t="n">
-        <v>0.02914792205987955</v>
+        <v>0.01354868317982921</v>
       </c>
       <c r="L18" s="12" t="n">
-        <v>789842.25</v>
+        <v>686760.25</v>
       </c>
       <c r="M18" s="12" t="n">
-        <v>600233.75</v>
+        <v>596777.25</v>
       </c>
       <c r="N18" s="13" t="n">
-        <v>-189608.5</v>
+        <v>-89983</v>
       </c>
       <c r="O18" s="14" t="n">
-        <v>-0.2400586952647823</v>
+        <v>-0.1310253469096384</v>
       </c>
       <c r="P18" s="10" t="inlineStr">
         <is>
@@ -1675,7 +1675,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AI18"/>
+  <dimension ref="A1:Z18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1684,12 +1684,12 @@
           <t>NAICS 5182 — Data Processing &amp; Hosting</t>
         </is>
       </c>
-      <c r="M1" s="3" t="inlineStr">
+      <c r="J1" s="3" t="inlineStr">
         <is>
           <t>NAICS 51 — Information Sector</t>
         </is>
       </c>
-      <c r="Y1" s="4" t="inlineStr">
+      <c r="S1" s="4" t="inlineStr">
         <is>
           <t>NAICS 517 — Telecommunications</t>
         </is>
@@ -1708,155 +1708,110 @@
       </c>
       <c r="C2" s="15" t="inlineStr">
         <is>
-          <t>2016</t>
+          <t>2019</t>
         </is>
       </c>
       <c r="D2" s="15" t="inlineStr">
         <is>
-          <t>2017</t>
+          <t>2020</t>
         </is>
       </c>
       <c r="E2" s="15" t="inlineStr">
         <is>
-          <t>2018</t>
+          <t>2021</t>
         </is>
       </c>
       <c r="F2" s="15" t="inlineStr">
         <is>
+          <t>2022</t>
+        </is>
+      </c>
+      <c r="G2" s="15" t="inlineStr">
+        <is>
+          <t>2023</t>
+        </is>
+      </c>
+      <c r="H2" s="15" t="inlineStr">
+        <is>
+          <t>2024</t>
+        </is>
+      </c>
+      <c r="J2" s="15" t="inlineStr">
+        <is>
+          <t>State</t>
+        </is>
+      </c>
+      <c r="K2" s="15" t="inlineStr">
+        <is>
+          <t>State Name</t>
+        </is>
+      </c>
+      <c r="L2" s="15" t="inlineStr">
+        <is>
           <t>2019</t>
         </is>
       </c>
-      <c r="G2" s="15" t="inlineStr">
+      <c r="M2" s="15" t="inlineStr">
         <is>
           <t>2020</t>
         </is>
       </c>
-      <c r="H2" s="15" t="inlineStr">
+      <c r="N2" s="15" t="inlineStr">
         <is>
           <t>2021</t>
         </is>
       </c>
-      <c r="I2" s="15" t="inlineStr">
+      <c r="O2" s="15" t="inlineStr">
         <is>
           <t>2022</t>
         </is>
       </c>
-      <c r="J2" s="15" t="inlineStr">
+      <c r="P2" s="15" t="inlineStr">
         <is>
           <t>2023</t>
         </is>
       </c>
-      <c r="K2" s="15" t="inlineStr">
+      <c r="Q2" s="15" t="inlineStr">
         <is>
           <t>2024</t>
         </is>
       </c>
-      <c r="M2" s="15" t="inlineStr">
+      <c r="S2" s="15" t="inlineStr">
         <is>
           <t>State</t>
         </is>
       </c>
-      <c r="N2" s="15" t="inlineStr">
+      <c r="T2" s="15" t="inlineStr">
         <is>
           <t>State Name</t>
         </is>
       </c>
-      <c r="O2" s="15" t="inlineStr">
-        <is>
-          <t>2016</t>
-        </is>
-      </c>
-      <c r="P2" s="15" t="inlineStr">
-        <is>
-          <t>2017</t>
-        </is>
-      </c>
-      <c r="Q2" s="15" t="inlineStr">
-        <is>
-          <t>2018</t>
-        </is>
-      </c>
-      <c r="R2" s="15" t="inlineStr">
+      <c r="U2" s="15" t="inlineStr">
         <is>
           <t>2019</t>
         </is>
       </c>
-      <c r="S2" s="15" t="inlineStr">
+      <c r="V2" s="15" t="inlineStr">
         <is>
           <t>2020</t>
         </is>
       </c>
-      <c r="T2" s="15" t="inlineStr">
+      <c r="W2" s="15" t="inlineStr">
         <is>
           <t>2021</t>
         </is>
       </c>
-      <c r="U2" s="15" t="inlineStr">
+      <c r="X2" s="15" t="inlineStr">
         <is>
           <t>2022</t>
         </is>
       </c>
-      <c r="V2" s="15" t="inlineStr">
+      <c r="Y2" s="15" t="inlineStr">
         <is>
           <t>2023</t>
         </is>
       </c>
-      <c r="W2" s="15" t="inlineStr">
-        <is>
-          <t>2024</t>
-        </is>
-      </c>
-      <c r="Y2" s="15" t="inlineStr">
-        <is>
-          <t>State</t>
-        </is>
-      </c>
       <c r="Z2" s="15" t="inlineStr">
-        <is>
-          <t>State Name</t>
-        </is>
-      </c>
-      <c r="AA2" s="15" t="inlineStr">
-        <is>
-          <t>2016</t>
-        </is>
-      </c>
-      <c r="AB2" s="15" t="inlineStr">
-        <is>
-          <t>2017</t>
-        </is>
-      </c>
-      <c r="AC2" s="15" t="inlineStr">
-        <is>
-          <t>2018</t>
-        </is>
-      </c>
-      <c r="AD2" s="15" t="inlineStr">
-        <is>
-          <t>2019</t>
-        </is>
-      </c>
-      <c r="AE2" s="15" t="inlineStr">
-        <is>
-          <t>2020</t>
-        </is>
-      </c>
-      <c r="AF2" s="15" t="inlineStr">
-        <is>
-          <t>2021</t>
-        </is>
-      </c>
-      <c r="AG2" s="15" t="inlineStr">
-        <is>
-          <t>2022</t>
-        </is>
-      </c>
-      <c r="AH2" s="15" t="inlineStr">
-        <is>
-          <t>2023</t>
-        </is>
-      </c>
-      <c r="AI2" s="15" t="inlineStr">
         <is>
           <t>2024</t>
         </is>
@@ -1874,104 +1829,77 @@
         </is>
       </c>
       <c r="C3" s="12" t="n">
-        <v>33241.5</v>
+        <v>36459.75</v>
       </c>
       <c r="D3" s="12" t="n">
-        <v>33959.5</v>
+        <v>38276.5</v>
       </c>
       <c r="E3" s="12" t="n">
-        <v>34883.5</v>
+        <v>39565</v>
       </c>
       <c r="F3" s="12" t="n">
-        <v>36459.75</v>
+        <v>45712.5</v>
       </c>
       <c r="G3" s="12" t="n">
-        <v>38276.5</v>
+        <v>47499.5</v>
       </c>
       <c r="H3" s="12" t="n">
-        <v>39565</v>
-      </c>
-      <c r="I3" s="12" t="n">
-        <v>45712.5</v>
-      </c>
-      <c r="J3" s="12" t="n">
-        <v>47499.5</v>
-      </c>
-      <c r="K3" s="12" t="n">
         <v>47316</v>
       </c>
-      <c r="M3" s="10" t="inlineStr">
+      <c r="J3" s="10" t="inlineStr">
         <is>
           <t>TX</t>
         </is>
       </c>
-      <c r="N3" s="10" t="inlineStr">
+      <c r="K3" s="10" t="inlineStr">
         <is>
           <t>Texas</t>
         </is>
       </c>
+      <c r="L3" s="12" t="n">
+        <v>207845.5</v>
+      </c>
+      <c r="M3" s="12" t="n">
+        <v>200111.25</v>
+      </c>
+      <c r="N3" s="12" t="n">
+        <v>206513.25</v>
+      </c>
       <c r="O3" s="12" t="n">
-        <v>204296.75</v>
+        <v>229987</v>
       </c>
       <c r="P3" s="12" t="n">
-        <v>203093</v>
+        <v>236486.25</v>
       </c>
       <c r="Q3" s="12" t="n">
-        <v>203936.75</v>
-      </c>
-      <c r="R3" s="12" t="n">
-        <v>207845.5</v>
-      </c>
-      <c r="S3" s="12" t="n">
-        <v>200111.25</v>
-      </c>
-      <c r="T3" s="12" t="n">
-        <v>206513.25</v>
+        <v>227371.75</v>
+      </c>
+      <c r="S3" s="10" t="inlineStr">
+        <is>
+          <t>TX</t>
+        </is>
+      </c>
+      <c r="T3" s="10" t="inlineStr">
+        <is>
+          <t>Texas</t>
+        </is>
       </c>
       <c r="U3" s="12" t="n">
-        <v>229987</v>
+        <v>76834.5</v>
       </c>
       <c r="V3" s="12" t="n">
-        <v>236486.25</v>
+        <v>76599</v>
       </c>
       <c r="W3" s="12" t="n">
-        <v>227371.75</v>
-      </c>
-      <c r="Y3" s="10" t="inlineStr">
-        <is>
-          <t>TX</t>
-        </is>
-      </c>
-      <c r="Z3" s="10" t="inlineStr">
-        <is>
-          <t>Texas</t>
-        </is>
-      </c>
-      <c r="AA3" s="12" t="n">
-        <v>81601.25</v>
-      </c>
-      <c r="AB3" s="12" t="n">
-        <v>80724.25</v>
-      </c>
-      <c r="AC3" s="12" t="n">
-        <v>78621.5</v>
-      </c>
-      <c r="AD3" s="12" t="n">
-        <v>76834.5</v>
-      </c>
-      <c r="AE3" s="12" t="n">
-        <v>76599</v>
-      </c>
-      <c r="AF3" s="12" t="n">
         <v>77669.75</v>
       </c>
-      <c r="AG3" s="12" t="n">
+      <c r="X3" s="12" t="n">
         <v>79860</v>
       </c>
-      <c r="AH3" s="12" t="n">
+      <c r="Y3" s="12" t="n">
         <v>80930</v>
       </c>
-      <c r="AI3" s="12" t="n">
+      <c r="Z3" s="12" t="n">
         <v>78831.25</v>
       </c>
     </row>
@@ -1987,104 +1915,77 @@
         </is>
       </c>
       <c r="C4" s="12" t="n">
-        <v>11038.75</v>
+        <v>13353.25</v>
       </c>
       <c r="D4" s="12" t="n">
-        <v>10868.25</v>
+        <v>14283.75</v>
       </c>
       <c r="E4" s="12" t="n">
-        <v>10620.5</v>
+        <v>14990</v>
       </c>
       <c r="F4" s="12" t="n">
-        <v>13353.25</v>
+        <v>17217.75</v>
       </c>
       <c r="G4" s="12" t="n">
-        <v>14283.75</v>
+        <v>18386.75</v>
       </c>
       <c r="H4" s="12" t="n">
-        <v>14990</v>
-      </c>
-      <c r="I4" s="12" t="n">
-        <v>17217.75</v>
-      </c>
-      <c r="J4" s="12" t="n">
-        <v>18386.75</v>
-      </c>
-      <c r="K4" s="12" t="n">
         <v>19382.75</v>
       </c>
-      <c r="M4" s="10" t="inlineStr">
+      <c r="J4" s="10" t="inlineStr">
         <is>
           <t>VA</t>
         </is>
       </c>
-      <c r="N4" s="10" t="inlineStr">
+      <c r="K4" s="10" t="inlineStr">
         <is>
           <t>Virginia</t>
         </is>
       </c>
+      <c r="L4" s="12" t="n">
+        <v>68727.25</v>
+      </c>
+      <c r="M4" s="12" t="n">
+        <v>67137.25</v>
+      </c>
+      <c r="N4" s="12" t="n">
+        <v>67084</v>
+      </c>
       <c r="O4" s="12" t="n">
-        <v>69401.25</v>
+        <v>70814.75</v>
       </c>
       <c r="P4" s="12" t="n">
-        <v>68800.25</v>
+        <v>72327.5</v>
       </c>
       <c r="Q4" s="12" t="n">
-        <v>68490</v>
-      </c>
-      <c r="R4" s="12" t="n">
-        <v>68727.25</v>
-      </c>
-      <c r="S4" s="12" t="n">
-        <v>67137.25</v>
-      </c>
-      <c r="T4" s="12" t="n">
-        <v>67084</v>
+        <v>71449.25</v>
+      </c>
+      <c r="S4" s="10" t="inlineStr">
+        <is>
+          <t>VA</t>
+        </is>
+      </c>
+      <c r="T4" s="10" t="inlineStr">
+        <is>
+          <t>Virginia</t>
+        </is>
       </c>
       <c r="U4" s="12" t="n">
-        <v>70814.75</v>
+        <v>22017.75</v>
       </c>
       <c r="V4" s="12" t="n">
-        <v>72327.5</v>
+        <v>21502.25</v>
       </c>
       <c r="W4" s="12" t="n">
-        <v>71449.25</v>
-      </c>
-      <c r="Y4" s="10" t="inlineStr">
-        <is>
-          <t>VA</t>
-        </is>
-      </c>
-      <c r="Z4" s="10" t="inlineStr">
-        <is>
-          <t>Virginia</t>
-        </is>
-      </c>
-      <c r="AA4" s="12" t="n">
-        <v>25559</v>
-      </c>
-      <c r="AB4" s="12" t="n">
-        <v>25374</v>
-      </c>
-      <c r="AC4" s="12" t="n">
-        <v>24899.25</v>
-      </c>
-      <c r="AD4" s="12" t="n">
-        <v>22017.75</v>
-      </c>
-      <c r="AE4" s="12" t="n">
-        <v>21502.25</v>
-      </c>
-      <c r="AF4" s="12" t="n">
         <v>20458.75</v>
       </c>
-      <c r="AG4" s="12" t="n">
+      <c r="X4" s="12" t="n">
         <v>19879.25</v>
       </c>
-      <c r="AH4" s="12" t="n">
+      <c r="Y4" s="12" t="n">
         <v>19770.5</v>
       </c>
-      <c r="AI4" s="12" t="n">
+      <c r="Z4" s="12" t="n">
         <v>18775.5</v>
       </c>
     </row>
@@ -2100,104 +2001,77 @@
         </is>
       </c>
       <c r="C5" s="12" t="n">
-        <v>3948.75</v>
+        <v>5658.25</v>
       </c>
       <c r="D5" s="12" t="n">
-        <v>4631.75</v>
+        <v>6345.25</v>
       </c>
       <c r="E5" s="12" t="n">
-        <v>4987.75</v>
+        <v>7194.5</v>
       </c>
       <c r="F5" s="12" t="n">
-        <v>5658.25</v>
+        <v>8049.5</v>
       </c>
       <c r="G5" s="12" t="n">
-        <v>6345.25</v>
+        <v>8278.75</v>
       </c>
       <c r="H5" s="12" t="n">
-        <v>7194.5</v>
-      </c>
-      <c r="I5" s="12" t="n">
-        <v>8049.5</v>
-      </c>
-      <c r="J5" s="12" t="n">
-        <v>8278.75</v>
-      </c>
-      <c r="K5" s="12" t="n">
         <v>8055</v>
       </c>
-      <c r="M5" s="10" t="inlineStr">
+      <c r="J5" s="10" t="inlineStr">
         <is>
           <t>OR</t>
         </is>
       </c>
-      <c r="N5" s="10" t="inlineStr">
+      <c r="K5" s="10" t="inlineStr">
         <is>
           <t>Oregon</t>
         </is>
       </c>
+      <c r="L5" s="12" t="n">
+        <v>36636.25</v>
+      </c>
+      <c r="M5" s="12" t="n">
+        <v>35255.25</v>
+      </c>
+      <c r="N5" s="12" t="n">
+        <v>37081</v>
+      </c>
       <c r="O5" s="12" t="n">
-        <v>34785.5</v>
+        <v>39219</v>
       </c>
       <c r="P5" s="12" t="n">
-        <v>35821.75</v>
+        <v>39565.75</v>
       </c>
       <c r="Q5" s="12" t="n">
-        <v>35834</v>
-      </c>
-      <c r="R5" s="12" t="n">
-        <v>36636.25</v>
-      </c>
-      <c r="S5" s="12" t="n">
-        <v>35255.25</v>
-      </c>
-      <c r="T5" s="12" t="n">
-        <v>37081</v>
+        <v>37579.5</v>
+      </c>
+      <c r="S5" s="10" t="inlineStr">
+        <is>
+          <t>OR</t>
+        </is>
+      </c>
+      <c r="T5" s="10" t="inlineStr">
+        <is>
+          <t>Oregon</t>
+        </is>
       </c>
       <c r="U5" s="12" t="n">
-        <v>39219</v>
+        <v>5179.25</v>
       </c>
       <c r="V5" s="12" t="n">
-        <v>39565.75</v>
+        <v>4895</v>
       </c>
       <c r="W5" s="12" t="n">
-        <v>37579.5</v>
-      </c>
-      <c r="Y5" s="10" t="inlineStr">
-        <is>
-          <t>OR</t>
-        </is>
-      </c>
-      <c r="Z5" s="10" t="inlineStr">
-        <is>
-          <t>Oregon</t>
-        </is>
-      </c>
-      <c r="AA5" s="12" t="n">
-        <v>5546.25</v>
-      </c>
-      <c r="AB5" s="12" t="n">
-        <v>5920.25</v>
-      </c>
-      <c r="AC5" s="12" t="n">
-        <v>5524.5</v>
-      </c>
-      <c r="AD5" s="12" t="n">
-        <v>5179.25</v>
-      </c>
-      <c r="AE5" s="12" t="n">
-        <v>4895</v>
-      </c>
-      <c r="AF5" s="12" t="n">
         <v>4645.5</v>
       </c>
-      <c r="AG5" s="12" t="n">
+      <c r="X5" s="12" t="n">
         <v>4321.75</v>
       </c>
-      <c r="AH5" s="12" t="n">
+      <c r="Y5" s="12" t="n">
         <v>4274.5</v>
       </c>
-      <c r="AI5" s="12" t="n">
+      <c r="Z5" s="12" t="n">
         <v>3963.75</v>
       </c>
     </row>
@@ -2213,104 +2087,77 @@
         </is>
       </c>
       <c r="C6" s="12" t="n">
-        <v>38885.5</v>
+        <v>51296.75</v>
       </c>
       <c r="D6" s="12" t="n">
-        <v>43195</v>
+        <v>54064.75</v>
       </c>
       <c r="E6" s="12" t="n">
-        <v>48080.25</v>
+        <v>54887.75</v>
       </c>
       <c r="F6" s="12" t="n">
-        <v>51296.75</v>
+        <v>70387.75</v>
       </c>
       <c r="G6" s="12" t="n">
-        <v>54064.75</v>
+        <v>80032.25</v>
       </c>
       <c r="H6" s="12" t="n">
-        <v>54887.75</v>
-      </c>
-      <c r="I6" s="12" t="n">
-        <v>70387.75</v>
-      </c>
-      <c r="J6" s="12" t="n">
-        <v>80032.25</v>
-      </c>
-      <c r="K6" s="12" t="n">
         <v>76245.75</v>
       </c>
-      <c r="M6" s="10" t="inlineStr">
+      <c r="J6" s="10" t="inlineStr">
         <is>
           <t>CA</t>
         </is>
       </c>
-      <c r="N6" s="10" t="inlineStr">
+      <c r="K6" s="10" t="inlineStr">
         <is>
           <t>California</t>
         </is>
       </c>
+      <c r="L6" s="12" t="n">
+        <v>734265.75</v>
+      </c>
+      <c r="M6" s="12" t="n">
+        <v>696680</v>
+      </c>
+      <c r="N6" s="12" t="n">
+        <v>739907.5</v>
+      </c>
       <c r="O6" s="12" t="n">
-        <v>671800.5</v>
+        <v>788877.5</v>
       </c>
       <c r="P6" s="12" t="n">
-        <v>679598.75</v>
+        <v>762161.75</v>
       </c>
       <c r="Q6" s="12" t="n">
-        <v>705676.75</v>
-      </c>
-      <c r="R6" s="12" t="n">
-        <v>734265.75</v>
-      </c>
-      <c r="S6" s="12" t="n">
-        <v>696680</v>
-      </c>
-      <c r="T6" s="12" t="n">
-        <v>739907.5</v>
+        <v>730032.5</v>
+      </c>
+      <c r="S6" s="10" t="inlineStr">
+        <is>
+          <t>CA</t>
+        </is>
+      </c>
+      <c r="T6" s="10" t="inlineStr">
+        <is>
+          <t>California</t>
+        </is>
       </c>
       <c r="U6" s="12" t="n">
-        <v>788877.5</v>
+        <v>63919</v>
       </c>
       <c r="V6" s="12" t="n">
-        <v>762161.75</v>
+        <v>59045.5</v>
       </c>
       <c r="W6" s="12" t="n">
-        <v>730032.5</v>
-      </c>
-      <c r="Y6" s="10" t="inlineStr">
-        <is>
-          <t>CA</t>
-        </is>
-      </c>
-      <c r="Z6" s="10" t="inlineStr">
-        <is>
-          <t>California</t>
-        </is>
-      </c>
-      <c r="AA6" s="12" t="n">
-        <v>76721</v>
-      </c>
-      <c r="AB6" s="12" t="n">
-        <v>71865.75</v>
-      </c>
-      <c r="AC6" s="12" t="n">
-        <v>67811.5</v>
-      </c>
-      <c r="AD6" s="12" t="n">
-        <v>63919</v>
-      </c>
-      <c r="AE6" s="12" t="n">
-        <v>59045.5</v>
-      </c>
-      <c r="AF6" s="12" t="n">
         <v>58098.25</v>
       </c>
-      <c r="AG6" s="12" t="n">
+      <c r="X6" s="12" t="n">
         <v>55342</v>
       </c>
-      <c r="AH6" s="12" t="n">
+      <c r="Y6" s="12" t="n">
         <v>53592</v>
       </c>
-      <c r="AI6" s="12" t="n">
+      <c r="Z6" s="12" t="n">
         <v>50936.5</v>
       </c>
     </row>
@@ -2326,104 +2173,77 @@
         </is>
       </c>
       <c r="C7" s="12" t="n">
-        <v>9607.25</v>
+        <v>10552.75</v>
       </c>
       <c r="D7" s="12" t="n">
-        <v>9653.5</v>
+        <v>10947.75</v>
       </c>
       <c r="E7" s="12" t="n">
-        <v>10267.5</v>
+        <v>11923.5</v>
       </c>
       <c r="F7" s="12" t="n">
-        <v>10552.75</v>
+        <v>14183</v>
       </c>
       <c r="G7" s="12" t="n">
-        <v>10947.75</v>
+        <v>15248.25</v>
       </c>
       <c r="H7" s="12" t="n">
-        <v>11923.5</v>
-      </c>
-      <c r="I7" s="12" t="n">
-        <v>14183</v>
-      </c>
-      <c r="J7" s="12" t="n">
-        <v>15248.25</v>
-      </c>
-      <c r="K7" s="12" t="n">
         <v>15356</v>
       </c>
-      <c r="M7" s="10" t="inlineStr">
+      <c r="J7" s="10" t="inlineStr">
         <is>
           <t>IL</t>
         </is>
       </c>
-      <c r="N7" s="10" t="inlineStr">
+      <c r="K7" s="10" t="inlineStr">
         <is>
           <t>Illinois</t>
         </is>
       </c>
+      <c r="L7" s="12" t="n">
+        <v>97058.5</v>
+      </c>
+      <c r="M7" s="12" t="n">
+        <v>89376.75</v>
+      </c>
+      <c r="N7" s="12" t="n">
+        <v>88267.75</v>
+      </c>
       <c r="O7" s="12" t="n">
-        <v>102705.5</v>
+        <v>95712.75</v>
       </c>
       <c r="P7" s="12" t="n">
-        <v>97428.25</v>
+        <v>94024</v>
       </c>
       <c r="Q7" s="12" t="n">
-        <v>96082.75</v>
-      </c>
-      <c r="R7" s="12" t="n">
-        <v>97058.5</v>
-      </c>
-      <c r="S7" s="12" t="n">
-        <v>89376.75</v>
-      </c>
-      <c r="T7" s="12" t="n">
-        <v>88267.75</v>
+        <v>89958.75</v>
+      </c>
+      <c r="S7" s="10" t="inlineStr">
+        <is>
+          <t>IL</t>
+        </is>
+      </c>
+      <c r="T7" s="10" t="inlineStr">
+        <is>
+          <t>Illinois</t>
+        </is>
       </c>
       <c r="U7" s="12" t="n">
-        <v>95712.75</v>
+        <v>25112.25</v>
       </c>
       <c r="V7" s="12" t="n">
-        <v>94024</v>
+        <v>23157.75</v>
       </c>
       <c r="W7" s="12" t="n">
-        <v>89958.75</v>
-      </c>
-      <c r="Y7" s="10" t="inlineStr">
-        <is>
-          <t>IL</t>
-        </is>
-      </c>
-      <c r="Z7" s="10" t="inlineStr">
-        <is>
-          <t>Illinois</t>
-        </is>
-      </c>
-      <c r="AA7" s="12" t="n">
-        <v>31955.25</v>
-      </c>
-      <c r="AB7" s="12" t="n">
-        <v>28459.75</v>
-      </c>
-      <c r="AC7" s="12" t="n">
-        <v>26679.5</v>
-      </c>
-      <c r="AD7" s="12" t="n">
-        <v>25112.25</v>
-      </c>
-      <c r="AE7" s="12" t="n">
-        <v>23157.75</v>
-      </c>
-      <c r="AF7" s="12" t="n">
         <v>21370.25</v>
       </c>
-      <c r="AG7" s="12" t="n">
+      <c r="X7" s="12" t="n">
         <v>21078.5</v>
       </c>
-      <c r="AH7" s="12" t="n">
+      <c r="Y7" s="12" t="n">
         <v>19850</v>
       </c>
-      <c r="AI7" s="12" t="n">
+      <c r="Z7" s="12" t="n">
         <v>18228.5</v>
       </c>
     </row>
@@ -2439,104 +2259,77 @@
         </is>
       </c>
       <c r="C8" s="12" t="n">
-        <v>9064.75</v>
+        <v>12587</v>
       </c>
       <c r="D8" s="12" t="n">
-        <v>10911.5</v>
+        <v>15097.25</v>
       </c>
       <c r="E8" s="12" t="n">
-        <v>11826.75</v>
+        <v>18416.75</v>
       </c>
       <c r="F8" s="12" t="n">
-        <v>12587</v>
+        <v>21791.5</v>
       </c>
       <c r="G8" s="12" t="n">
-        <v>15097.25</v>
+        <v>24943</v>
       </c>
       <c r="H8" s="12" t="n">
-        <v>18416.75</v>
-      </c>
-      <c r="I8" s="12" t="n">
-        <v>21791.5</v>
-      </c>
-      <c r="J8" s="12" t="n">
-        <v>24943</v>
-      </c>
-      <c r="K8" s="12" t="n">
         <v>23823</v>
       </c>
-      <c r="M8" s="10" t="inlineStr">
+      <c r="J8" s="10" t="inlineStr">
         <is>
           <t>GA</t>
         </is>
       </c>
-      <c r="N8" s="10" t="inlineStr">
+      <c r="K8" s="10" t="inlineStr">
         <is>
           <t>Georgia</t>
         </is>
       </c>
+      <c r="L8" s="12" t="n">
+        <v>121740.5</v>
+      </c>
+      <c r="M8" s="12" t="n">
+        <v>114851.75</v>
+      </c>
+      <c r="N8" s="12" t="n">
+        <v>124045.75</v>
+      </c>
       <c r="O8" s="12" t="n">
-        <v>115357.5</v>
+        <v>137027.5</v>
       </c>
       <c r="P8" s="12" t="n">
-        <v>121798.25</v>
+        <v>130510.5</v>
       </c>
       <c r="Q8" s="12" t="n">
-        <v>122387.5</v>
-      </c>
-      <c r="R8" s="12" t="n">
-        <v>121740.5</v>
-      </c>
-      <c r="S8" s="12" t="n">
-        <v>114851.75</v>
-      </c>
-      <c r="T8" s="12" t="n">
-        <v>124045.75</v>
+        <v>128801.75</v>
+      </c>
+      <c r="S8" s="10" t="inlineStr">
+        <is>
+          <t>GA</t>
+        </is>
+      </c>
+      <c r="T8" s="10" t="inlineStr">
+        <is>
+          <t>Georgia</t>
+        </is>
       </c>
       <c r="U8" s="12" t="n">
-        <v>137027.5</v>
+        <v>40880</v>
       </c>
       <c r="V8" s="12" t="n">
-        <v>130510.5</v>
+        <v>38734.25</v>
       </c>
       <c r="W8" s="12" t="n">
-        <v>128801.75</v>
-      </c>
-      <c r="Y8" s="10" t="inlineStr">
-        <is>
-          <t>GA</t>
-        </is>
-      </c>
-      <c r="Z8" s="10" t="inlineStr">
-        <is>
-          <t>Georgia</t>
-        </is>
-      </c>
-      <c r="AA8" s="12" t="n">
-        <v>47632.5</v>
-      </c>
-      <c r="AB8" s="12" t="n">
-        <v>45902.75</v>
-      </c>
-      <c r="AC8" s="12" t="n">
-        <v>43783.25</v>
-      </c>
-      <c r="AD8" s="12" t="n">
-        <v>40880</v>
-      </c>
-      <c r="AE8" s="12" t="n">
-        <v>38734.25</v>
-      </c>
-      <c r="AF8" s="12" t="n">
         <v>38233.75</v>
       </c>
-      <c r="AG8" s="12" t="n">
+      <c r="X8" s="12" t="n">
         <v>39138.25</v>
       </c>
-      <c r="AH8" s="12" t="n">
+      <c r="Y8" s="12" t="n">
         <v>36492.5</v>
       </c>
-      <c r="AI8" s="12" t="n">
+      <c r="Z8" s="12" t="n">
         <v>34363</v>
       </c>
     </row>
@@ -2552,104 +2345,77 @@
         </is>
       </c>
       <c r="C9" s="12" t="n">
-        <v>6641.5</v>
+        <v>8350</v>
       </c>
       <c r="D9" s="12" t="n">
-        <v>7076.75</v>
+        <v>8732</v>
       </c>
       <c r="E9" s="12" t="n">
-        <v>7611.5</v>
+        <v>8915.5</v>
       </c>
       <c r="F9" s="12" t="n">
-        <v>8350</v>
+        <v>11418.5</v>
       </c>
       <c r="G9" s="12" t="n">
-        <v>8732</v>
+        <v>11535.5</v>
       </c>
       <c r="H9" s="12" t="n">
-        <v>8915.5</v>
-      </c>
-      <c r="I9" s="12" t="n">
-        <v>11418.5</v>
-      </c>
-      <c r="J9" s="12" t="n">
-        <v>11535.5</v>
-      </c>
-      <c r="K9" s="12" t="n">
         <v>11627</v>
       </c>
-      <c r="M9" s="10" t="inlineStr">
+      <c r="J9" s="10" t="inlineStr">
         <is>
           <t>OH</t>
         </is>
       </c>
-      <c r="N9" s="10" t="inlineStr">
+      <c r="K9" s="10" t="inlineStr">
         <is>
           <t>Ohio</t>
         </is>
       </c>
+      <c r="L9" s="12" t="n">
+        <v>72140.5</v>
+      </c>
+      <c r="M9" s="12" t="n">
+        <v>67123.75</v>
+      </c>
+      <c r="N9" s="12" t="n">
+        <v>66514.75</v>
+      </c>
       <c r="O9" s="12" t="n">
-        <v>73169.75</v>
+        <v>70752.25</v>
       </c>
       <c r="P9" s="12" t="n">
-        <v>74088.75</v>
+        <v>69683.75</v>
       </c>
       <c r="Q9" s="12" t="n">
-        <v>73321.5</v>
-      </c>
-      <c r="R9" s="12" t="n">
-        <v>72140.5</v>
-      </c>
-      <c r="S9" s="12" t="n">
-        <v>67123.75</v>
-      </c>
-      <c r="T9" s="12" t="n">
-        <v>66514.75</v>
+        <v>67882</v>
+      </c>
+      <c r="S9" s="10" t="inlineStr">
+        <is>
+          <t>OH</t>
+        </is>
+      </c>
+      <c r="T9" s="10" t="inlineStr">
+        <is>
+          <t>Ohio</t>
+        </is>
       </c>
       <c r="U9" s="12" t="n">
-        <v>70752.25</v>
+        <v>24094</v>
       </c>
       <c r="V9" s="12" t="n">
-        <v>69683.75</v>
+        <v>22424</v>
       </c>
       <c r="W9" s="12" t="n">
-        <v>67882</v>
-      </c>
-      <c r="Y9" s="10" t="inlineStr">
-        <is>
-          <t>OH</t>
-        </is>
-      </c>
-      <c r="Z9" s="10" t="inlineStr">
-        <is>
-          <t>Ohio</t>
-        </is>
-      </c>
-      <c r="AA9" s="12" t="n">
-        <v>24497.5</v>
-      </c>
-      <c r="AB9" s="12" t="n">
-        <v>25767.25</v>
-      </c>
-      <c r="AC9" s="12" t="n">
-        <v>25263</v>
-      </c>
-      <c r="AD9" s="12" t="n">
-        <v>24094</v>
-      </c>
-      <c r="AE9" s="12" t="n">
-        <v>22424</v>
-      </c>
-      <c r="AF9" s="12" t="n">
         <v>21644.25</v>
       </c>
-      <c r="AG9" s="12" t="n">
+      <c r="X9" s="12" t="n">
         <v>21481</v>
       </c>
-      <c r="AH9" s="12" t="n">
+      <c r="Y9" s="12" t="n">
         <v>21398.25</v>
       </c>
-      <c r="AI9" s="12" t="n">
+      <c r="Z9" s="12" t="n">
         <v>20227</v>
       </c>
     </row>
@@ -2665,104 +2431,77 @@
         </is>
       </c>
       <c r="C10" s="12" t="n">
-        <v>8529.25</v>
+        <v>9851</v>
       </c>
       <c r="D10" s="12" t="n">
-        <v>8998.25</v>
+        <v>9956.75</v>
       </c>
       <c r="E10" s="12" t="n">
-        <v>9473.75</v>
+        <v>11760.25</v>
       </c>
       <c r="F10" s="12" t="n">
-        <v>9851</v>
+        <v>12901.75</v>
       </c>
       <c r="G10" s="12" t="n">
-        <v>9956.75</v>
+        <v>12743</v>
       </c>
       <c r="H10" s="12" t="n">
-        <v>11760.25</v>
-      </c>
-      <c r="I10" s="12" t="n">
-        <v>12901.75</v>
-      </c>
-      <c r="J10" s="12" t="n">
-        <v>12743</v>
-      </c>
-      <c r="K10" s="12" t="n">
         <v>11946.5</v>
       </c>
-      <c r="M10" s="10" t="inlineStr">
+      <c r="J10" s="10" t="inlineStr">
         <is>
           <t>AZ</t>
         </is>
       </c>
-      <c r="N10" s="10" t="inlineStr">
+      <c r="K10" s="10" t="inlineStr">
         <is>
           <t>Arizona</t>
         </is>
       </c>
+      <c r="L10" s="12" t="n">
+        <v>49423.5</v>
+      </c>
+      <c r="M10" s="12" t="n">
+        <v>47135.75</v>
+      </c>
+      <c r="N10" s="12" t="n">
+        <v>48059.5</v>
+      </c>
       <c r="O10" s="12" t="n">
-        <v>45130.5</v>
+        <v>51826.5</v>
       </c>
       <c r="P10" s="12" t="n">
-        <v>46442</v>
+        <v>52109.25</v>
       </c>
       <c r="Q10" s="12" t="n">
-        <v>48123.5</v>
-      </c>
-      <c r="R10" s="12" t="n">
-        <v>49423.5</v>
-      </c>
-      <c r="S10" s="12" t="n">
-        <v>47135.75</v>
-      </c>
-      <c r="T10" s="12" t="n">
-        <v>48059.5</v>
+        <v>50194.75</v>
+      </c>
+      <c r="S10" s="10" t="inlineStr">
+        <is>
+          <t>AZ</t>
+        </is>
+      </c>
+      <c r="T10" s="10" t="inlineStr">
+        <is>
+          <t>Arizona</t>
+        </is>
       </c>
       <c r="U10" s="12" t="n">
-        <v>51826.5</v>
+        <v>16073.75</v>
       </c>
       <c r="V10" s="12" t="n">
-        <v>52109.25</v>
+        <v>15472.25</v>
       </c>
       <c r="W10" s="12" t="n">
-        <v>50194.75</v>
-      </c>
-      <c r="Y10" s="10" t="inlineStr">
-        <is>
-          <t>AZ</t>
-        </is>
-      </c>
-      <c r="Z10" s="10" t="inlineStr">
-        <is>
-          <t>Arizona</t>
-        </is>
-      </c>
-      <c r="AA10" s="12" t="n">
-        <v>15105.5</v>
-      </c>
-      <c r="AB10" s="12" t="n">
-        <v>15963.75</v>
-      </c>
-      <c r="AC10" s="12" t="n">
-        <v>16396.5</v>
-      </c>
-      <c r="AD10" s="12" t="n">
-        <v>16073.75</v>
-      </c>
-      <c r="AE10" s="12" t="n">
-        <v>15472.25</v>
-      </c>
-      <c r="AF10" s="12" t="n">
         <v>14236.5</v>
       </c>
-      <c r="AG10" s="12" t="n">
+      <c r="X10" s="12" t="n">
         <v>13268.25</v>
       </c>
-      <c r="AH10" s="12" t="n">
+      <c r="Y10" s="12" t="n">
         <v>12240.75</v>
       </c>
-      <c r="AI10" s="12" t="n">
+      <c r="Z10" s="12" t="n">
         <v>11782.75</v>
       </c>
     </row>
@@ -2778,104 +2517,77 @@
         </is>
       </c>
       <c r="C11" s="12" t="n">
-        <v>3091.25</v>
+        <v>3459.25</v>
       </c>
       <c r="D11" s="12" t="n">
-        <v>3053.25</v>
+        <v>3277.5</v>
       </c>
       <c r="E11" s="12" t="n">
-        <v>3543.5</v>
+        <v>3296.5</v>
       </c>
       <c r="F11" s="12" t="n">
-        <v>3459.25</v>
+        <v>3422.75</v>
       </c>
       <c r="G11" s="12" t="n">
-        <v>3277.5</v>
+        <v>3239.75</v>
       </c>
       <c r="H11" s="12" t="n">
-        <v>3296.5</v>
-      </c>
-      <c r="I11" s="12" t="n">
-        <v>3422.75</v>
-      </c>
-      <c r="J11" s="12" t="n">
-        <v>3239.75</v>
-      </c>
-      <c r="K11" s="12" t="n">
         <v>3348.5</v>
       </c>
-      <c r="M11" s="10" t="inlineStr">
+      <c r="J11" s="10" t="inlineStr">
         <is>
           <t>IA</t>
         </is>
       </c>
-      <c r="N11" s="10" t="inlineStr">
+      <c r="K11" s="10" t="inlineStr">
         <is>
           <t>Iowa</t>
         </is>
       </c>
+      <c r="L11" s="12" t="n">
+        <v>20899.5</v>
+      </c>
+      <c r="M11" s="12" t="n">
+        <v>18801</v>
+      </c>
+      <c r="N11" s="12" t="n">
+        <v>18030.25</v>
+      </c>
       <c r="O11" s="12" t="n">
-        <v>22338.5</v>
+        <v>17894.75</v>
       </c>
       <c r="P11" s="12" t="n">
-        <v>21605</v>
+        <v>18067.25</v>
       </c>
       <c r="Q11" s="12" t="n">
-        <v>21428.5</v>
-      </c>
-      <c r="R11" s="12" t="n">
-        <v>20899.5</v>
-      </c>
-      <c r="S11" s="12" t="n">
-        <v>18801</v>
-      </c>
-      <c r="T11" s="12" t="n">
-        <v>18030.25</v>
+        <v>17900.5</v>
+      </c>
+      <c r="S11" s="10" t="inlineStr">
+        <is>
+          <t>IA</t>
+        </is>
+      </c>
+      <c r="T11" s="10" t="inlineStr">
+        <is>
+          <t>Iowa</t>
+        </is>
       </c>
       <c r="U11" s="12" t="n">
-        <v>17894.75</v>
+        <v>5687.75</v>
       </c>
       <c r="V11" s="12" t="n">
-        <v>18067.25</v>
+        <v>5429</v>
       </c>
       <c r="W11" s="12" t="n">
-        <v>17900.5</v>
-      </c>
-      <c r="Y11" s="10" t="inlineStr">
-        <is>
-          <t>IA</t>
-        </is>
-      </c>
-      <c r="Z11" s="10" t="inlineStr">
-        <is>
-          <t>Iowa</t>
-        </is>
-      </c>
-      <c r="AA11" s="12" t="n">
-        <v>6507.5</v>
-      </c>
-      <c r="AB11" s="12" t="n">
-        <v>6248</v>
-      </c>
-      <c r="AC11" s="12" t="n">
-        <v>6168</v>
-      </c>
-      <c r="AD11" s="12" t="n">
-        <v>5687.75</v>
-      </c>
-      <c r="AE11" s="12" t="n">
-        <v>5429</v>
-      </c>
-      <c r="AF11" s="12" t="n">
         <v>4965.25</v>
       </c>
-      <c r="AG11" s="12" t="n">
+      <c r="X11" s="12" t="n">
         <v>4993.75</v>
       </c>
-      <c r="AH11" s="12" t="n">
+      <c r="Y11" s="12" t="n">
         <v>5114</v>
       </c>
-      <c r="AI11" s="12" t="n">
+      <c r="Z11" s="12" t="n">
         <v>5047</v>
       </c>
     </row>
@@ -2891,104 +2603,77 @@
         </is>
       </c>
       <c r="C12" s="12" t="n">
-        <v>9019</v>
+        <v>13382.25</v>
       </c>
       <c r="D12" s="12" t="n">
-        <v>11096.25</v>
+        <v>13599.25</v>
       </c>
       <c r="E12" s="12" t="n">
-        <v>11518.25</v>
+        <v>15220</v>
       </c>
       <c r="F12" s="12" t="n">
-        <v>13382.25</v>
+        <v>24861</v>
       </c>
       <c r="G12" s="12" t="n">
-        <v>13599.25</v>
+        <v>23492.25</v>
       </c>
       <c r="H12" s="12" t="n">
-        <v>15220</v>
-      </c>
-      <c r="I12" s="12" t="n">
-        <v>24861</v>
-      </c>
-      <c r="J12" s="12" t="n">
-        <v>23492.25</v>
-      </c>
-      <c r="K12" s="12" t="n">
         <v>22821</v>
       </c>
-      <c r="M12" s="10" t="inlineStr">
+      <c r="J12" s="10" t="inlineStr">
         <is>
           <t>WA</t>
         </is>
       </c>
-      <c r="N12" s="10" t="inlineStr">
+      <c r="K12" s="10" t="inlineStr">
         <is>
           <t>Washington</t>
         </is>
       </c>
+      <c r="L12" s="12" t="n">
+        <v>148345.25</v>
+      </c>
+      <c r="M12" s="12" t="n">
+        <v>156172.5</v>
+      </c>
+      <c r="N12" s="12" t="n">
+        <v>166091</v>
+      </c>
       <c r="O12" s="12" t="n">
-        <v>127577.75</v>
+        <v>182054.75</v>
       </c>
       <c r="P12" s="12" t="n">
-        <v>134427.25</v>
+        <v>182074.75</v>
       </c>
       <c r="Q12" s="12" t="n">
-        <v>140317</v>
-      </c>
-      <c r="R12" s="12" t="n">
-        <v>148345.25</v>
-      </c>
-      <c r="S12" s="12" t="n">
-        <v>156172.5</v>
-      </c>
-      <c r="T12" s="12" t="n">
-        <v>166091</v>
+        <v>173738.5</v>
+      </c>
+      <c r="S12" s="10" t="inlineStr">
+        <is>
+          <t>WA</t>
+        </is>
+      </c>
+      <c r="T12" s="10" t="inlineStr">
+        <is>
+          <t>Washington</t>
+        </is>
       </c>
       <c r="U12" s="12" t="n">
-        <v>182054.75</v>
+        <v>20125</v>
       </c>
       <c r="V12" s="12" t="n">
-        <v>182074.75</v>
+        <v>18870</v>
       </c>
       <c r="W12" s="12" t="n">
-        <v>173738.5</v>
-      </c>
-      <c r="Y12" s="10" t="inlineStr">
-        <is>
-          <t>WA</t>
-        </is>
-      </c>
-      <c r="Z12" s="10" t="inlineStr">
-        <is>
-          <t>Washington</t>
-        </is>
-      </c>
-      <c r="AA12" s="12" t="n">
-        <v>21661</v>
-      </c>
-      <c r="AB12" s="12" t="n">
-        <v>21462.5</v>
-      </c>
-      <c r="AC12" s="12" t="n">
-        <v>20766.75</v>
-      </c>
-      <c r="AD12" s="12" t="n">
-        <v>20125</v>
-      </c>
-      <c r="AE12" s="12" t="n">
-        <v>18870</v>
-      </c>
-      <c r="AF12" s="12" t="n">
         <v>18800.5</v>
       </c>
-      <c r="AG12" s="12" t="n">
+      <c r="X12" s="12" t="n">
         <v>18180</v>
       </c>
-      <c r="AH12" s="12" t="n">
+      <c r="Y12" s="12" t="n">
         <v>17278.75</v>
       </c>
-      <c r="AI12" s="12" t="n">
+      <c r="Z12" s="12" t="n">
         <v>16161.75</v>
       </c>
     </row>
@@ -3004,104 +2689,77 @@
         </is>
       </c>
       <c r="C13" s="12" t="n">
-        <v>14147.75</v>
+        <v>10570.5</v>
       </c>
       <c r="D13" s="12" t="n">
-        <v>14806.5</v>
+        <v>10019.5</v>
       </c>
       <c r="E13" s="12" t="n">
-        <v>15338.25</v>
+        <v>10799</v>
       </c>
       <c r="F13" s="12" t="n">
-        <v>10570.5</v>
+        <v>10986</v>
       </c>
       <c r="G13" s="12" t="n">
-        <v>10019.5</v>
+        <v>11534.75</v>
       </c>
       <c r="H13" s="12" t="n">
-        <v>10799</v>
-      </c>
-      <c r="I13" s="12" t="n">
-        <v>10986</v>
-      </c>
-      <c r="J13" s="12" t="n">
-        <v>11534.75</v>
-      </c>
-      <c r="K13" s="12" t="n">
         <v>11933.5</v>
       </c>
-      <c r="M13" s="10" t="inlineStr">
+      <c r="J13" s="10" t="inlineStr">
         <is>
           <t>NC</t>
         </is>
       </c>
-      <c r="N13" s="10" t="inlineStr">
+      <c r="K13" s="10" t="inlineStr">
         <is>
           <t>North Carolina</t>
         </is>
       </c>
+      <c r="L13" s="12" t="n">
+        <v>74603.25</v>
+      </c>
+      <c r="M13" s="12" t="n">
+        <v>72188.5</v>
+      </c>
+      <c r="N13" s="12" t="n">
+        <v>74278.25</v>
+      </c>
       <c r="O13" s="12" t="n">
-        <v>79755.25</v>
+        <v>78786.25</v>
       </c>
       <c r="P13" s="12" t="n">
-        <v>76986.25</v>
+        <v>83036.75</v>
       </c>
       <c r="Q13" s="12" t="n">
-        <v>77403.25</v>
-      </c>
-      <c r="R13" s="12" t="n">
-        <v>74603.25</v>
-      </c>
-      <c r="S13" s="12" t="n">
-        <v>72188.5</v>
-      </c>
-      <c r="T13" s="12" t="n">
-        <v>74278.25</v>
+        <v>82062</v>
+      </c>
+      <c r="S13" s="10" t="inlineStr">
+        <is>
+          <t>NC</t>
+        </is>
+      </c>
+      <c r="T13" s="10" t="inlineStr">
+        <is>
+          <t>North Carolina</t>
+        </is>
       </c>
       <c r="U13" s="12" t="n">
-        <v>78786.25</v>
+        <v>23721.5</v>
       </c>
       <c r="V13" s="12" t="n">
-        <v>83036.75</v>
+        <v>24499.5</v>
       </c>
       <c r="W13" s="12" t="n">
-        <v>82062</v>
-      </c>
-      <c r="Y13" s="10" t="inlineStr">
-        <is>
-          <t>NC</t>
-        </is>
-      </c>
-      <c r="Z13" s="10" t="inlineStr">
-        <is>
-          <t>North Carolina</t>
-        </is>
-      </c>
-      <c r="AA13" s="12" t="n">
-        <v>26572.25</v>
-      </c>
-      <c r="AB13" s="12" t="n">
-        <v>24369.25</v>
-      </c>
-      <c r="AC13" s="12" t="n">
-        <v>23543</v>
-      </c>
-      <c r="AD13" s="12" t="n">
-        <v>23721.5</v>
-      </c>
-      <c r="AE13" s="12" t="n">
-        <v>24499.5</v>
-      </c>
-      <c r="AF13" s="12" t="n">
         <v>24076.5</v>
       </c>
-      <c r="AG13" s="12" t="n">
+      <c r="X13" s="12" t="n">
         <v>23294.25</v>
       </c>
-      <c r="AH13" s="12" t="n">
+      <c r="Y13" s="12" t="n">
         <v>23454</v>
       </c>
-      <c r="AI13" s="12" t="n">
+      <c r="Z13" s="12" t="n">
         <v>21836.75</v>
       </c>
     </row>
@@ -3117,104 +2775,77 @@
         </is>
       </c>
       <c r="C14" s="12" t="n">
-        <v>8716.75</v>
+        <v>9784.5</v>
       </c>
       <c r="D14" s="12" t="n">
-        <v>8952</v>
+        <v>10903.75</v>
       </c>
       <c r="E14" s="12" t="n">
-        <v>9253.25</v>
+        <v>11935.25</v>
       </c>
       <c r="F14" s="12" t="n">
-        <v>9784.5</v>
+        <v>13510.75</v>
       </c>
       <c r="G14" s="12" t="n">
-        <v>10903.75</v>
+        <v>14193.5</v>
       </c>
       <c r="H14" s="12" t="n">
-        <v>11935.25</v>
-      </c>
-      <c r="I14" s="12" t="n">
-        <v>13510.75</v>
-      </c>
-      <c r="J14" s="12" t="n">
-        <v>14193.5</v>
-      </c>
-      <c r="K14" s="12" t="n">
         <v>13362.75</v>
       </c>
-      <c r="M14" s="10" t="inlineStr">
+      <c r="J14" s="10" t="inlineStr">
         <is>
           <t>PA</t>
         </is>
       </c>
-      <c r="N14" s="10" t="inlineStr">
+      <c r="K14" s="10" t="inlineStr">
         <is>
           <t>Pennsylvania</t>
         </is>
       </c>
+      <c r="L14" s="12" t="n">
+        <v>90644.25</v>
+      </c>
+      <c r="M14" s="12" t="n">
+        <v>87876.25</v>
+      </c>
+      <c r="N14" s="12" t="n">
+        <v>87547.25</v>
+      </c>
       <c r="O14" s="12" t="n">
-        <v>88182.75</v>
+        <v>95130.75</v>
       </c>
       <c r="P14" s="12" t="n">
-        <v>87181.25</v>
+        <v>95409.25</v>
       </c>
       <c r="Q14" s="12" t="n">
-        <v>90058.25</v>
-      </c>
-      <c r="R14" s="12" t="n">
-        <v>90644.25</v>
-      </c>
-      <c r="S14" s="12" t="n">
-        <v>87876.25</v>
-      </c>
-      <c r="T14" s="12" t="n">
-        <v>87547.25</v>
+        <v>93065</v>
+      </c>
+      <c r="S14" s="10" t="inlineStr">
+        <is>
+          <t>PA</t>
+        </is>
+      </c>
+      <c r="T14" s="10" t="inlineStr">
+        <is>
+          <t>Pennsylvania</t>
+        </is>
       </c>
       <c r="U14" s="12" t="n">
-        <v>95130.75</v>
+        <v>28645</v>
       </c>
       <c r="V14" s="12" t="n">
-        <v>95409.25</v>
+        <v>29083.5</v>
       </c>
       <c r="W14" s="12" t="n">
-        <v>93065</v>
-      </c>
-      <c r="Y14" s="10" t="inlineStr">
-        <is>
-          <t>PA</t>
-        </is>
-      </c>
-      <c r="Z14" s="10" t="inlineStr">
-        <is>
-          <t>Pennsylvania</t>
-        </is>
-      </c>
-      <c r="AA14" s="12" t="n">
-        <v>29335.5</v>
-      </c>
-      <c r="AB14" s="12" t="n">
-        <v>29077.5</v>
-      </c>
-      <c r="AC14" s="12" t="n">
-        <v>29211.5</v>
-      </c>
-      <c r="AD14" s="12" t="n">
-        <v>28645</v>
-      </c>
-      <c r="AE14" s="12" t="n">
-        <v>29083.5</v>
-      </c>
-      <c r="AF14" s="12" t="n">
         <v>27091</v>
       </c>
-      <c r="AG14" s="12" t="n">
+      <c r="X14" s="12" t="n">
         <v>28233.75</v>
       </c>
-      <c r="AH14" s="12" t="n">
+      <c r="Y14" s="12" t="n">
         <v>27628.75</v>
       </c>
-      <c r="AI14" s="12" t="n">
+      <c r="Z14" s="12" t="n">
         <v>26767.25</v>
       </c>
     </row>
@@ -3230,104 +2861,77 @@
         </is>
       </c>
       <c r="C15" s="12" t="n">
-        <v>518</v>
+        <v>487.25</v>
       </c>
       <c r="D15" s="12" t="n">
-        <v>518</v>
+        <v>456</v>
       </c>
       <c r="E15" s="12" t="n">
-        <v>504</v>
+        <v>462.25</v>
       </c>
       <c r="F15" s="12" t="n">
-        <v>487.25</v>
+        <v>462.5</v>
       </c>
       <c r="G15" s="12" t="n">
-        <v>456</v>
+        <v>360</v>
       </c>
       <c r="H15" s="12" t="n">
-        <v>462.25</v>
-      </c>
-      <c r="I15" s="12" t="n">
-        <v>462.5</v>
-      </c>
-      <c r="J15" s="12" t="n">
-        <v>360</v>
-      </c>
-      <c r="K15" s="12" t="n">
         <v>313.5</v>
       </c>
-      <c r="M15" s="10" t="inlineStr">
+      <c r="J15" s="10" t="inlineStr">
         <is>
           <t>ND</t>
         </is>
       </c>
-      <c r="N15" s="10" t="inlineStr">
+      <c r="K15" s="10" t="inlineStr">
         <is>
           <t>North Dakota</t>
         </is>
       </c>
+      <c r="L15" s="12" t="n">
+        <v>6253.75</v>
+      </c>
+      <c r="M15" s="12" t="n">
+        <v>5963.75</v>
+      </c>
+      <c r="N15" s="12" t="n">
+        <v>5969.75</v>
+      </c>
       <c r="O15" s="12" t="n">
-        <v>6896.75</v>
+        <v>6080.75</v>
       </c>
       <c r="P15" s="12" t="n">
-        <v>6822</v>
+        <v>5842.25</v>
       </c>
       <c r="Q15" s="12" t="n">
-        <v>6553.25</v>
-      </c>
-      <c r="R15" s="12" t="n">
-        <v>6253.75</v>
-      </c>
-      <c r="S15" s="12" t="n">
-        <v>5963.75</v>
-      </c>
-      <c r="T15" s="12" t="n">
-        <v>5969.75</v>
+        <v>5539</v>
+      </c>
+      <c r="S15" s="10" t="inlineStr">
+        <is>
+          <t>ND</t>
+        </is>
+      </c>
+      <c r="T15" s="10" t="inlineStr">
+        <is>
+          <t>North Dakota</t>
+        </is>
       </c>
       <c r="U15" s="12" t="n">
-        <v>6080.75</v>
+        <v>1777.75</v>
       </c>
       <c r="V15" s="12" t="n">
-        <v>5842.25</v>
+        <v>1798.75</v>
       </c>
       <c r="W15" s="12" t="n">
-        <v>5539</v>
-      </c>
-      <c r="Y15" s="10" t="inlineStr">
-        <is>
-          <t>ND</t>
-        </is>
-      </c>
-      <c r="Z15" s="10" t="inlineStr">
-        <is>
-          <t>North Dakota</t>
-        </is>
-      </c>
-      <c r="AA15" s="12" t="n">
-        <v>1871.5</v>
-      </c>
-      <c r="AB15" s="12" t="n">
-        <v>1803.75</v>
-      </c>
-      <c r="AC15" s="12" t="n">
-        <v>1778.5</v>
-      </c>
-      <c r="AD15" s="12" t="n">
-        <v>1777.75</v>
-      </c>
-      <c r="AE15" s="12" t="n">
-        <v>1798.75</v>
-      </c>
-      <c r="AF15" s="12" t="n">
         <v>1886.75</v>
       </c>
-      <c r="AG15" s="12" t="n">
+      <c r="X15" s="12" t="n">
         <v>2019.5</v>
       </c>
-      <c r="AH15" s="12" t="n">
+      <c r="Y15" s="12" t="n">
         <v>2034.75</v>
       </c>
-      <c r="AI15" s="12" t="n">
+      <c r="Z15" s="12" t="n">
         <v>1985.5</v>
       </c>
     </row>
@@ -3343,104 +2947,77 @@
         </is>
       </c>
       <c r="C16" s="12" t="n">
-        <v>1669</v>
+        <v>2342.5</v>
       </c>
       <c r="D16" s="12" t="n">
-        <v>1799.25</v>
+        <v>2197.25</v>
       </c>
       <c r="E16" s="12" t="n">
-        <v>2373.25</v>
+        <v>2481.5</v>
       </c>
       <c r="F16" s="12" t="n">
-        <v>2342.5</v>
+        <v>2911.5</v>
       </c>
       <c r="G16" s="12" t="n">
-        <v>2197.25</v>
+        <v>3065.75</v>
       </c>
       <c r="H16" s="12" t="n">
-        <v>2481.5</v>
-      </c>
-      <c r="I16" s="12" t="n">
-        <v>2911.5</v>
-      </c>
-      <c r="J16" s="12" t="n">
-        <v>3065.75</v>
-      </c>
-      <c r="K16" s="12" t="n">
         <v>2935.25</v>
       </c>
-      <c r="M16" s="10" t="inlineStr">
+      <c r="J16" s="10" t="inlineStr">
         <is>
           <t>NV</t>
         </is>
       </c>
-      <c r="N16" s="10" t="inlineStr">
+      <c r="K16" s="10" t="inlineStr">
         <is>
           <t>Nevada</t>
         </is>
       </c>
+      <c r="L16" s="12" t="n">
+        <v>16906.75</v>
+      </c>
+      <c r="M16" s="12" t="n">
+        <v>14973.25</v>
+      </c>
+      <c r="N16" s="12" t="n">
+        <v>16171.75</v>
+      </c>
       <c r="O16" s="12" t="n">
-        <v>14868.5</v>
+        <v>19745.25</v>
       </c>
       <c r="P16" s="12" t="n">
-        <v>15492.75</v>
+        <v>21314.5</v>
       </c>
       <c r="Q16" s="12" t="n">
-        <v>16574.75</v>
-      </c>
-      <c r="R16" s="12" t="n">
-        <v>16906.75</v>
-      </c>
-      <c r="S16" s="12" t="n">
-        <v>14973.25</v>
-      </c>
-      <c r="T16" s="12" t="n">
-        <v>16171.75</v>
+        <v>21858.75</v>
+      </c>
+      <c r="S16" s="10" t="inlineStr">
+        <is>
+          <t>NV</t>
+        </is>
+      </c>
+      <c r="T16" s="10" t="inlineStr">
+        <is>
+          <t>Nevada</t>
+        </is>
       </c>
       <c r="U16" s="12" t="n">
-        <v>19745.25</v>
+        <v>4065</v>
       </c>
       <c r="V16" s="12" t="n">
-        <v>21314.5</v>
+        <v>3860.75</v>
       </c>
       <c r="W16" s="12" t="n">
-        <v>21858.75</v>
-      </c>
-      <c r="Y16" s="10" t="inlineStr">
-        <is>
-          <t>NV</t>
-        </is>
-      </c>
-      <c r="Z16" s="10" t="inlineStr">
-        <is>
-          <t>Nevada</t>
-        </is>
-      </c>
-      <c r="AA16" s="12" t="n">
-        <v>3973.25</v>
-      </c>
-      <c r="AB16" s="12" t="n">
-        <v>4085.75</v>
-      </c>
-      <c r="AC16" s="12" t="n">
-        <v>4143.25</v>
-      </c>
-      <c r="AD16" s="12" t="n">
-        <v>4065</v>
-      </c>
-      <c r="AE16" s="12" t="n">
-        <v>3860.75</v>
-      </c>
-      <c r="AF16" s="12" t="n">
         <v>3921.25</v>
       </c>
-      <c r="AG16" s="12" t="n">
+      <c r="X16" s="12" t="n">
         <v>4039</v>
       </c>
-      <c r="AH16" s="12" t="n">
+      <c r="Y16" s="12" t="n">
         <v>3837.25</v>
       </c>
-      <c r="AI16" s="12" t="n">
+      <c r="Z16" s="12" t="n">
         <v>3633.25</v>
       </c>
     </row>
@@ -3456,104 +3033,77 @@
         </is>
       </c>
       <c r="C17" s="12" t="n">
-        <v>4642.25</v>
+        <v>4020.5</v>
       </c>
       <c r="D17" s="12" t="n">
-        <v>4542.5</v>
+        <v>3595.5</v>
       </c>
       <c r="E17" s="12" t="n">
-        <v>4279.25</v>
+        <v>2246</v>
       </c>
       <c r="F17" s="12" t="n">
-        <v>4020.5</v>
+        <v>2224.75</v>
       </c>
       <c r="G17" s="12" t="n">
-        <v>3595.5</v>
+        <v>2062</v>
       </c>
       <c r="H17" s="12" t="n">
-        <v>2246</v>
-      </c>
-      <c r="I17" s="12" t="n">
-        <v>2224.75</v>
-      </c>
-      <c r="J17" s="12" t="n">
-        <v>2062</v>
-      </c>
-      <c r="K17" s="12" t="n">
         <v>1887.75</v>
       </c>
-      <c r="M17" s="10" t="inlineStr">
+      <c r="J17" s="10" t="inlineStr">
         <is>
           <t>NE</t>
         </is>
       </c>
-      <c r="N17" s="10" t="inlineStr">
+      <c r="K17" s="10" t="inlineStr">
         <is>
           <t>Nebraska</t>
         </is>
       </c>
+      <c r="L17" s="12" t="n">
+        <v>17148.75</v>
+      </c>
+      <c r="M17" s="12" t="n">
+        <v>16399.5</v>
+      </c>
+      <c r="N17" s="12" t="n">
+        <v>17785.75</v>
+      </c>
       <c r="O17" s="12" t="n">
-        <v>18448.75</v>
+        <v>18493.75</v>
       </c>
       <c r="P17" s="12" t="n">
-        <v>18220.5</v>
+        <v>17813.5</v>
       </c>
       <c r="Q17" s="12" t="n">
-        <v>17546.25</v>
-      </c>
-      <c r="R17" s="12" t="n">
-        <v>17148.75</v>
-      </c>
-      <c r="S17" s="12" t="n">
-        <v>16399.5</v>
-      </c>
-      <c r="T17" s="12" t="n">
-        <v>17785.75</v>
+        <v>18053</v>
+      </c>
+      <c r="S17" s="10" t="inlineStr">
+        <is>
+          <t>NE</t>
+        </is>
+      </c>
+      <c r="T17" s="10" t="inlineStr">
+        <is>
+          <t>Nebraska</t>
+        </is>
       </c>
       <c r="U17" s="12" t="n">
-        <v>18493.75</v>
+        <v>3318.75</v>
       </c>
       <c r="V17" s="12" t="n">
-        <v>17813.5</v>
+        <v>3102.75</v>
       </c>
       <c r="W17" s="12" t="n">
-        <v>18053</v>
-      </c>
-      <c r="Y17" s="10" t="inlineStr">
-        <is>
-          <t>NE</t>
-        </is>
-      </c>
-      <c r="Z17" s="10" t="inlineStr">
-        <is>
-          <t>Nebraska</t>
-        </is>
-      </c>
-      <c r="AA17" s="12" t="n">
-        <v>3551.25</v>
-      </c>
-      <c r="AB17" s="12" t="n">
-        <v>3768.75</v>
-      </c>
-      <c r="AC17" s="12" t="n">
-        <v>3560.5</v>
-      </c>
-      <c r="AD17" s="12" t="n">
-        <v>3318.75</v>
-      </c>
-      <c r="AE17" s="12" t="n">
-        <v>3102.75</v>
-      </c>
-      <c r="AF17" s="12" t="n">
         <v>2930.25</v>
       </c>
-      <c r="AG17" s="12" t="n">
+      <c r="X17" s="12" t="n">
         <v>3056</v>
       </c>
-      <c r="AH17" s="12" t="n">
+      <c r="Y17" s="12" t="n">
         <v>3165</v>
       </c>
-      <c r="AI17" s="12" t="n">
+      <c r="Z17" s="12" t="n">
         <v>3071.25</v>
       </c>
     </row>
@@ -3565,116 +3115,89 @@
       </c>
       <c r="B18" s="10" t="inlineStr">
         <is>
-          <t>National</t>
+          <t>National (balanced, 48 units)</t>
         </is>
       </c>
       <c r="C18" s="12" t="n">
-        <v>300874.25</v>
+        <v>333652.25</v>
       </c>
       <c r="D18" s="12" t="n">
-        <v>314778.5</v>
+        <v>352638.75</v>
       </c>
       <c r="E18" s="12" t="n">
-        <v>333296.5</v>
+        <v>373671</v>
       </c>
       <c r="F18" s="12" t="n">
-        <v>341842.25</v>
+        <v>446404.25</v>
       </c>
       <c r="G18" s="12" t="n">
-        <v>361105.5</v>
+        <v>468579.75</v>
       </c>
       <c r="H18" s="12" t="n">
-        <v>382707.75</v>
-      </c>
-      <c r="I18" s="12" t="n">
-        <v>447021.25</v>
-      </c>
-      <c r="J18" s="12" t="n">
-        <v>469199</v>
-      </c>
-      <c r="K18" s="12" t="n">
-        <v>464954.8333333333</v>
-      </c>
-      <c r="M18" s="10" t="inlineStr">
+        <v>464389.0833333333</v>
+      </c>
+      <c r="J18" s="10" t="inlineStr">
         <is>
           <t>US</t>
         </is>
       </c>
-      <c r="N18" s="10" t="inlineStr">
-        <is>
-          <t>National</t>
-        </is>
+      <c r="K18" s="10" t="inlineStr">
+        <is>
+          <t>National (balanced, 48 units)</t>
+        </is>
+      </c>
+      <c r="L18" s="12" t="n">
+        <v>3062567</v>
+      </c>
+      <c r="M18" s="12" t="n">
+        <v>2911072</v>
+      </c>
+      <c r="N18" s="12" t="n">
+        <v>2985662</v>
       </c>
       <c r="O18" s="12" t="n">
-        <v>3026759.5</v>
+        <v>3230944.5</v>
       </c>
       <c r="P18" s="12" t="n">
-        <v>3030089.25</v>
+        <v>3194080</v>
       </c>
       <c r="Q18" s="12" t="n">
-        <v>3091112</v>
-      </c>
-      <c r="R18" s="12" t="n">
-        <v>3131159.25</v>
-      </c>
-      <c r="S18" s="12" t="n">
-        <v>2973666.25</v>
-      </c>
-      <c r="T18" s="12" t="n">
-        <v>3049186</v>
+        <v>3104060.75</v>
+      </c>
+      <c r="S18" s="10" t="inlineStr">
+        <is>
+          <t>US</t>
+        </is>
+      </c>
+      <c r="T18" s="10" t="inlineStr">
+        <is>
+          <t>National (balanced, 48 units)</t>
+        </is>
       </c>
       <c r="U18" s="12" t="n">
-        <v>3242481</v>
+        <v>686760.25</v>
       </c>
       <c r="V18" s="12" t="n">
-        <v>3205633.5</v>
+        <v>663073.75</v>
       </c>
       <c r="W18" s="12" t="n">
-        <v>3114983.25</v>
-      </c>
-      <c r="Y18" s="10" t="inlineStr">
-        <is>
-          <t>US</t>
-        </is>
-      </c>
-      <c r="Z18" s="10" t="inlineStr">
-        <is>
-          <t>National</t>
-        </is>
-      </c>
-      <c r="AA18" s="12" t="n">
-        <v>789842.25</v>
-      </c>
-      <c r="AB18" s="12" t="n">
-        <v>754820.25</v>
-      </c>
-      <c r="AC18" s="12" t="n">
-        <v>745926.25</v>
-      </c>
-      <c r="AD18" s="12" t="n">
-        <v>707118.25</v>
-      </c>
-      <c r="AE18" s="12" t="n">
-        <v>682331.5</v>
-      </c>
-      <c r="AF18" s="12" t="n">
-        <v>665629.5</v>
-      </c>
-      <c r="AG18" s="12" t="n">
-        <v>643462</v>
-      </c>
-      <c r="AH18" s="12" t="n">
-        <v>629190.5</v>
-      </c>
-      <c r="AI18" s="12" t="n">
-        <v>600233.75</v>
+        <v>647058</v>
+      </c>
+      <c r="X18" s="12" t="n">
+        <v>639912</v>
+      </c>
+      <c r="Y18" s="12" t="n">
+        <v>625654.5</v>
+      </c>
+      <c r="Z18" s="12" t="n">
+        <v>596777.25</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="3">
-    <mergeCell ref="A1:K1"/>
-    <mergeCell ref="M1:W1"/>
-    <mergeCell ref="Y1:AI1"/>
+    <mergeCell ref="J1:Q1"/>
+    <mergeCell ref="S1:Z1"/>
+    <mergeCell ref="A1:H1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -3805,28 +3328,28 @@
         <v>8.942662</v>
       </c>
       <c r="D3" s="13" t="n">
-        <v>14074.5</v>
+        <v>10856.25</v>
       </c>
       <c r="E3" s="14" t="n">
-        <v>0.4234014710527503</v>
+        <v>0.2977598584740707</v>
       </c>
       <c r="F3" s="13" t="n">
-        <v>-2770</v>
+        <v>1996.75</v>
       </c>
       <c r="G3" s="14" t="n">
-        <v>-0.03394555843200931</v>
+        <v>0.02598767480754088</v>
       </c>
       <c r="H3" s="13" t="n">
-        <v>23075</v>
+        <v>19526.25</v>
       </c>
       <c r="I3" s="14" t="n">
-        <v>0.1129484438690287</v>
+        <v>0.09394598391593756</v>
       </c>
       <c r="J3" s="13" t="n">
-        <v>11304.5</v>
+        <v>12853</v>
       </c>
       <c r="K3" s="18" t="n">
-        <v>5.081046931407943</v>
+        <v>5.436960060097658</v>
       </c>
     </row>
     <row r="4">
@@ -3844,28 +3367,28 @@
         <v>8.239623999999999</v>
       </c>
       <c r="D4" s="13" t="n">
-        <v>8344</v>
+        <v>6029.5</v>
       </c>
       <c r="E4" s="14" t="n">
-        <v>0.7558826859925263</v>
+        <v>0.4515380150899594</v>
       </c>
       <c r="F4" s="13" t="n">
-        <v>-6783.5</v>
+        <v>-3242.25</v>
       </c>
       <c r="G4" s="14" t="n">
-        <v>-0.2654055322978207</v>
+        <v>-0.1472561910276936</v>
       </c>
       <c r="H4" s="13" t="n">
-        <v>2048</v>
+        <v>2722</v>
       </c>
       <c r="I4" s="14" t="n">
-        <v>0.02950955494317465</v>
+        <v>0.03960583320298717</v>
       </c>
       <c r="J4" s="13" t="n">
-        <v>1560.5</v>
+        <v>2787.25</v>
       </c>
       <c r="K4" s="18" t="n">
-        <v>1.230043487874991</v>
+        <v>1.859665355848562</v>
       </c>
     </row>
     <row r="5">
@@ -3883,28 +3406,28 @@
         <v>4.588372000000001</v>
       </c>
       <c r="D5" s="13" t="n">
-        <v>4106.25</v>
+        <v>2396.75</v>
       </c>
       <c r="E5" s="14" t="n">
-        <v>1.03988603988604</v>
+        <v>0.4235850307073742</v>
       </c>
       <c r="F5" s="13" t="n">
-        <v>-1582.5</v>
+        <v>-1215.5</v>
       </c>
       <c r="G5" s="14" t="n">
-        <v>-0.2853279242731576</v>
+        <v>-0.2346864893565671</v>
       </c>
       <c r="H5" s="13" t="n">
-        <v>2794</v>
+        <v>943.25</v>
       </c>
       <c r="I5" s="14" t="n">
-        <v>0.08032082333156057</v>
+        <v>0.02574635777406258</v>
       </c>
       <c r="J5" s="13" t="n">
-        <v>2523.75</v>
+        <v>1181.25</v>
       </c>
       <c r="K5" s="18" t="n">
-        <v>2.59478672985782</v>
+        <v>1.971822295351707</v>
       </c>
     </row>
     <row r="6">
@@ -3922,28 +3445,28 @@
         <v>3.473613</v>
       </c>
       <c r="D6" s="13" t="n">
-        <v>37360.25</v>
+        <v>24949</v>
       </c>
       <c r="E6" s="14" t="n">
-        <v>0.9607758676113204</v>
+        <v>0.4863660953179295</v>
       </c>
       <c r="F6" s="13" t="n">
-        <v>-25784.5</v>
+        <v>-12982.5</v>
       </c>
       <c r="G6" s="14" t="n">
-        <v>-0.3360813858004979</v>
+        <v>-0.2031086218495283</v>
       </c>
       <c r="H6" s="13" t="n">
-        <v>58232</v>
+        <v>-4233.25</v>
       </c>
       <c r="I6" s="14" t="n">
-        <v>0.08668049517676751</v>
+        <v>-0.00576528320979155</v>
       </c>
       <c r="J6" s="13" t="n">
-        <v>11575.75</v>
+        <v>11966.5</v>
       </c>
       <c r="K6" s="18" t="n">
-        <v>1.448942193953732</v>
+        <v>1.921740804929713</v>
       </c>
     </row>
     <row r="7">
@@ -3961,28 +3484,28 @@
         <v>2.805081</v>
       </c>
       <c r="D7" s="13" t="n">
-        <v>5748.75</v>
+        <v>4803.25</v>
       </c>
       <c r="E7" s="14" t="n">
-        <v>0.5983762262874391</v>
+        <v>0.4551657150979602</v>
       </c>
       <c r="F7" s="13" t="n">
-        <v>-13726.75</v>
+        <v>-6883.75</v>
       </c>
       <c r="G7" s="14" t="n">
-        <v>-0.4295616526235908</v>
+        <v>-0.2741192047705801</v>
       </c>
       <c r="H7" s="13" t="n">
-        <v>-12746.75</v>
+        <v>-7099.75</v>
       </c>
       <c r="I7" s="14" t="n">
-        <v>-0.1241097117486405</v>
+        <v>-0.07314918322455015</v>
       </c>
       <c r="J7" s="13" t="n">
-        <v>-7978</v>
+        <v>-2080.5</v>
       </c>
       <c r="K7" s="18" t="n">
-        <v>0.4187990602291147</v>
+        <v>0.6977664790266933</v>
       </c>
     </row>
     <row r="8">
@@ -4000,28 +3523,28 @@
         <v>2.55925</v>
       </c>
       <c r="D8" s="13" t="n">
-        <v>14758.25</v>
+        <v>11236</v>
       </c>
       <c r="E8" s="14" t="n">
-        <v>1.628092335695965</v>
+        <v>0.8926670374195599</v>
       </c>
       <c r="F8" s="13" t="n">
-        <v>-13269.5</v>
+        <v>-6517</v>
       </c>
       <c r="G8" s="14" t="n">
-        <v>-0.278580800923739</v>
+        <v>-0.1594178082191781</v>
       </c>
       <c r="H8" s="13" t="n">
-        <v>13444.25</v>
+        <v>7061.25</v>
       </c>
       <c r="I8" s="14" t="n">
-        <v>0.1165442212253213</v>
+        <v>0.05800247247218469</v>
       </c>
       <c r="J8" s="13" t="n">
-        <v>1488.75</v>
+        <v>4719</v>
       </c>
       <c r="K8" s="18" t="n">
-        <v>1.112193375786578</v>
+        <v>1.724106183826914</v>
       </c>
     </row>
     <row r="9">
@@ -4039,28 +3562,28 @@
         <v>2.434877</v>
       </c>
       <c r="D9" s="13" t="n">
-        <v>4985.5</v>
+        <v>3277</v>
       </c>
       <c r="E9" s="14" t="n">
-        <v>0.7506587367311601</v>
+        <v>0.3924550898203593</v>
       </c>
       <c r="F9" s="13" t="n">
-        <v>-4270.5</v>
+        <v>-3867</v>
       </c>
       <c r="G9" s="14" t="n">
-        <v>-0.1743239106031228</v>
+        <v>-0.1604963891425251</v>
       </c>
       <c r="H9" s="13" t="n">
-        <v>-5287.75</v>
+        <v>-4258.5</v>
       </c>
       <c r="I9" s="14" t="n">
-        <v>-0.07226688624739049</v>
+        <v>-0.05903064159522044</v>
       </c>
       <c r="J9" s="13" t="n">
-        <v>715</v>
+        <v>-590</v>
       </c>
       <c r="K9" s="18" t="n">
-        <v>1.167427701674277</v>
+        <v>0.8474269459529351</v>
       </c>
     </row>
     <row r="10">
@@ -4078,28 +3601,28 @@
         <v>2.392509</v>
       </c>
       <c r="D10" s="13" t="n">
-        <v>3417.25</v>
+        <v>2095.5</v>
       </c>
       <c r="E10" s="14" t="n">
-        <v>0.4006507019960723</v>
+        <v>0.2127195208608263</v>
       </c>
       <c r="F10" s="13" t="n">
-        <v>-3322.75</v>
+        <v>-4291</v>
       </c>
       <c r="G10" s="14" t="n">
-        <v>-0.2199695475158055</v>
+        <v>-0.2669569951007077</v>
       </c>
       <c r="H10" s="13" t="n">
-        <v>5064.25</v>
+        <v>771.25</v>
       </c>
       <c r="I10" s="14" t="n">
-        <v>0.1122134698263924</v>
+        <v>0.01560492478274505</v>
       </c>
       <c r="J10" s="13" t="n">
-        <v>94.5</v>
+        <v>-2195.5</v>
       </c>
       <c r="K10" s="18" t="n">
-        <v>1.028440297945979</v>
+        <v>0.4883477044977861</v>
       </c>
     </row>
     <row r="11">
@@ -4117,28 +3640,28 @@
         <v>2.237543</v>
       </c>
       <c r="D11" s="13" t="n">
-        <v>257.25</v>
+        <v>-110.75</v>
       </c>
       <c r="E11" s="14" t="n">
-        <v>0.08321876263647392</v>
+        <v>-0.0320156103201561</v>
       </c>
       <c r="F11" s="13" t="n">
-        <v>-1460.5</v>
+        <v>-640.75</v>
       </c>
       <c r="G11" s="14" t="n">
-        <v>-0.2244333461390703</v>
+        <v>-0.1126543888180739</v>
       </c>
       <c r="H11" s="13" t="n">
-        <v>-4438</v>
+        <v>-2999</v>
       </c>
       <c r="I11" s="14" t="n">
-        <v>-0.1986704568346129</v>
+        <v>-0.1434962558912893</v>
       </c>
       <c r="J11" s="13" t="n">
-        <v>-1203.25</v>
+        <v>-751.5</v>
       </c>
       <c r="K11" s="18" t="n">
-        <v>0.1761383087983567</v>
+        <v>0.1728443230589153</v>
       </c>
     </row>
     <row r="12">
@@ -4156,28 +3679,28 @@
         <v>1.900304</v>
       </c>
       <c r="D12" s="13" t="n">
-        <v>13802</v>
+        <v>9438.75</v>
       </c>
       <c r="E12" s="14" t="n">
-        <v>1.530324869719481</v>
+        <v>0.705318612340974</v>
       </c>
       <c r="F12" s="13" t="n">
-        <v>-5499.25</v>
+        <v>-3963.25</v>
       </c>
       <c r="G12" s="14" t="n">
-        <v>-0.2538779373066802</v>
+        <v>-0.1969316770186335</v>
       </c>
       <c r="H12" s="13" t="n">
-        <v>46160.75</v>
+        <v>25393.25</v>
       </c>
       <c r="I12" s="14" t="n">
-        <v>0.3618244560669866</v>
+        <v>0.1711766976023836</v>
       </c>
       <c r="J12" s="13" t="n">
-        <v>8302.75</v>
+        <v>5475.5</v>
       </c>
       <c r="K12" s="18" t="n">
-        <v>2.509796790471428</v>
+        <v>2.38156815744654</v>
       </c>
     </row>
     <row r="13">
@@ -4195,28 +3718,28 @@
         <v>1.594719</v>
       </c>
       <c r="D13" s="13" t="n">
-        <v>-2214.25</v>
+        <v>1363</v>
       </c>
       <c r="E13" s="14" t="n">
-        <v>-0.1565089855277341</v>
+        <v>0.1289437585733882</v>
       </c>
       <c r="F13" s="13" t="n">
-        <v>-4735.5</v>
+        <v>-1884.75</v>
       </c>
       <c r="G13" s="14" t="n">
-        <v>-0.1782122326863551</v>
+        <v>-0.07945323862318994</v>
       </c>
       <c r="H13" s="13" t="n">
-        <v>2306.75</v>
+        <v>7458.75</v>
       </c>
       <c r="I13" s="14" t="n">
-        <v>0.02892286087749709</v>
+        <v>0.09997888831920862</v>
       </c>
       <c r="J13" s="13" t="n">
-        <v>-6949.75</v>
+        <v>-521.75</v>
       </c>
       <c r="K13" s="18" t="n">
-        <v>0.4675852602681871</v>
+        <v>0.7231728345934474</v>
       </c>
     </row>
     <row r="14">
@@ -4234,28 +3757,28 @@
         <v>1.512326</v>
       </c>
       <c r="D14" s="13" t="n">
-        <v>4646</v>
+        <v>3578.25</v>
       </c>
       <c r="E14" s="14" t="n">
-        <v>0.5329968164740299</v>
+        <v>0.3657059635137207</v>
       </c>
       <c r="F14" s="13" t="n">
-        <v>-2568.25</v>
+        <v>-1877.75</v>
       </c>
       <c r="G14" s="14" t="n">
-        <v>-0.08754751069523274</v>
+        <v>-0.06555245243497992</v>
       </c>
       <c r="H14" s="13" t="n">
-        <v>4882.25</v>
+        <v>2420.75</v>
       </c>
       <c r="I14" s="14" t="n">
-        <v>0.05536513660551525</v>
+        <v>0.02670605140425344</v>
       </c>
       <c r="J14" s="13" t="n">
-        <v>2077.75</v>
+        <v>1700.5</v>
       </c>
       <c r="K14" s="18" t="n">
-        <v>1.809013919984425</v>
+        <v>1.905605112501664</v>
       </c>
     </row>
     <row r="15">
@@ -4273,28 +3796,28 @@
         <v>1.468625</v>
       </c>
       <c r="D15" s="13" t="n">
-        <v>-204.5</v>
+        <v>-173.75</v>
       </c>
       <c r="E15" s="14" t="n">
-        <v>-0.3947876447876448</v>
+        <v>-0.3565931246793227</v>
       </c>
       <c r="F15" s="13" t="n">
-        <v>114</v>
+        <v>207.75</v>
       </c>
       <c r="G15" s="14" t="n">
-        <v>0.06091370558375635</v>
+        <v>0.1168612009562649</v>
       </c>
       <c r="H15" s="13" t="n">
-        <v>-1357.75</v>
+        <v>-714.75</v>
       </c>
       <c r="I15" s="14" t="n">
-        <v>-0.1968680900424113</v>
+        <v>-0.1142914251449131</v>
       </c>
       <c r="J15" s="13" t="n">
-        <v>-90.5</v>
+        <v>34</v>
       </c>
       <c r="K15" s="18" t="n">
-        <v>1.793859649122807</v>
+        <v>0.8363417569193743</v>
       </c>
     </row>
     <row r="16">
@@ -4312,28 +3835,28 @@
         <v>1.449626</v>
       </c>
       <c r="D16" s="13" t="n">
-        <v>1266.25</v>
+        <v>592.75</v>
       </c>
       <c r="E16" s="14" t="n">
-        <v>0.7586878370281606</v>
+        <v>0.2530416221985058</v>
       </c>
       <c r="F16" s="13" t="n">
-        <v>-340</v>
+        <v>-431.75</v>
       </c>
       <c r="G16" s="14" t="n">
-        <v>-0.08557226451897061</v>
+        <v>-0.1062115621156212</v>
       </c>
       <c r="H16" s="13" t="n">
-        <v>6990.25</v>
+        <v>4952</v>
       </c>
       <c r="I16" s="14" t="n">
-        <v>0.4701382116555133</v>
+        <v>0.2929007644875568</v>
       </c>
       <c r="J16" s="13" t="n">
-        <v>926.25</v>
+        <v>161</v>
       </c>
       <c r="K16" s="18" t="n">
-        <v>3.724264705882353</v>
+        <v>1.372900984365953</v>
       </c>
     </row>
     <row r="17">
@@ -4351,28 +3874,28 @@
         <v>1.256079</v>
       </c>
       <c r="D17" s="13" t="n">
-        <v>-2754.5</v>
+        <v>-2132.75</v>
       </c>
       <c r="E17" s="14" t="n">
-        <v>-0.5933545155905003</v>
+        <v>-0.5304688471583137</v>
       </c>
       <c r="F17" s="13" t="n">
-        <v>-480</v>
+        <v>-247.5</v>
       </c>
       <c r="G17" s="14" t="n">
-        <v>-0.1351636747624076</v>
+        <v>-0.07457627118644068</v>
       </c>
       <c r="H17" s="13" t="n">
-        <v>-395.75</v>
+        <v>904.25</v>
       </c>
       <c r="I17" s="14" t="n">
-        <v>-0.02145131783996206</v>
+        <v>0.0527297908010788</v>
       </c>
       <c r="J17" s="13" t="n">
-        <v>-3234.5</v>
+        <v>-2380.25</v>
       </c>
       <c r="K17" s="18" t="n">
-        <v>5.738541666666666</v>
+        <v>8.617171717171717</v>
       </c>
     </row>
     <row r="18">
@@ -4387,31 +3910,31 @@
         </is>
       </c>
       <c r="C18" s="11" t="n">
-        <v>56.613435</v>
+        <v>56.595705</v>
       </c>
       <c r="D18" s="13" t="n">
-        <v>164080.5833333333</v>
+        <v>130736.8333333333</v>
       </c>
       <c r="E18" s="14" t="n">
-        <v>0.5453460485014364</v>
+        <v>0.3918356112789089</v>
       </c>
       <c r="F18" s="13" t="n">
-        <v>-189608.5</v>
+        <v>-89983</v>
       </c>
       <c r="G18" s="14" t="n">
-        <v>-0.2400586952647823</v>
+        <v>-0.1310253469096384</v>
       </c>
       <c r="H18" s="13" t="n">
-        <v>88223.75</v>
+        <v>41493.75</v>
       </c>
       <c r="I18" s="14" t="n">
-        <v>0.02914792205987955</v>
+        <v>0.01354868317982921</v>
       </c>
       <c r="J18" s="13" t="n">
-        <v>-25527.91666666669</v>
+        <v>40753.83333333331</v>
       </c>
       <c r="K18" s="18" t="n">
-        <v>0.865365125157012</v>
+        <v>1.452905919266231</v>
       </c>
     </row>
   </sheetData>

</xml_diff>